<commit_message>
adding FASTA alignment and mapping
</commit_message>
<xml_diff>
--- a/data/proteins/pipeline.xlsx
+++ b/data/proteins/pipeline.xlsx
@@ -420,8 +420,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="65" customWidth="1" min="3" max="3"/>
+    <col width="71" customWidth="1" min="4" max="4"/>
+    <col width="82" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -436,25 +449,45 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>pdb_directory</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>fasta_directory</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>alignment_directory</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>pdb_sync_done</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>fasta_files_done</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
         <is>
           <t>sequence_alignment_done</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>numbering_check_done</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>modeller_done</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>protonation_done</t>
         </is>
@@ -471,15 +504,39 @@
           <t>10-200</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta/alignments</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>success</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -492,15 +549,39 @@
           <t>5-150</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2W8Y</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2W8Y/fasta</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2W8Y/fasta/alignments</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>success</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Dealing wir insertion codes
</commit_message>
<xml_diff>
--- a/data/proteins/pipeline.xlsx
+++ b/data/proteins/pipeline.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -432,8 +432,9 @@
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="25" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -479,15 +480,20 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>insertion_codes_done</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>numbering_check_done</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>modeller_done</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>protonation_done</t>
         </is>
@@ -534,9 +540,14 @@
           <t>success</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -579,9 +590,14 @@
           <t>success</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" s="1" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Adding rebuilding residues functionality
</commit_message>
<xml_diff>
--- a/data/proteins/pipeline.xlsx
+++ b/data/proteins/pipeline.xlsx
@@ -26,7 +26,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -37,6 +37,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
         <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+        <bgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -52,9 +58,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,23 +427,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:U3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
     <col width="65" customWidth="1" min="3" max="3"/>
     <col width="71" customWidth="1" min="4" max="4"/>
     <col width="82" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="25" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="15" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="76" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="26" customWidth="1" min="17" max="17"/>
+    <col width="91" customWidth="1" min="18" max="18"/>
+    <col width="112" customWidth="1" min="19" max="19"/>
+    <col width="15" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -467,45 +481,80 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>uniprot_id</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>components_directory</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>n_gaps</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>gap_sizes</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>pdb_sync_done</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>fasta_files_done</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>sequence_alignment_done</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>insertion_codes_done</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>numbering_check_done</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>modeller_done</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>has_metals</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>has_ligands</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>has_nonstandard_residues</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>filler_directory</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>filler_model_path</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>filler_status</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
         <is>
           <t>protonation_done</t>
         </is>
@@ -514,47 +563,47 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2AFX</t>
+          <t>1IOO</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>10-200</t>
+          <t>6-284</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1IOO</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1IOO/fasta</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta/alignments</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1IOO/fasta/alignments</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Q7SID5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>6|6</t>
-        </is>
-      </c>
-      <c r="H2" s="1" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="I2" s="1" t="inlineStr">
-        <is>
-          <t>success</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1IOO/components</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>none</t>
         </is>
       </c>
       <c r="J2" s="1" t="inlineStr">
@@ -567,50 +616,85 @@
           <t>success</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
+      <c r="L2" s="1" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="M2" s="1" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
       <c r="N2" t="inlineStr"/>
+      <c r="O2" s="1" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="Q2" s="1" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" s="1" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2W8Y</t>
+          <t>2P1T</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>5-150</t>
+          <t>229-458</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2W8Y</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2W8Y/fasta</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2W8Y/fasta/alignments</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta/alignments</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" s="1" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="I3" s="1" t="inlineStr">
-        <is>
-          <t>success</t>
+          <t>P19793</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/components</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>19</t>
         </is>
       </c>
       <c r="J3" s="1" t="inlineStr">
@@ -623,9 +707,48 @@
           <t>success</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
+      <c r="L3" s="1" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="M3" s="1" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
       <c r="N3" t="inlineStr"/>
+      <c r="O3" s="1" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="Q3" s="1" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta/alignments/filler/A</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta/alignments/filler/A/2P1T_protein_mod.pdb</t>
+        </is>
+      </c>
+      <c r="T3" s="1" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Adapting to AMBER naming convention
</commit_message>
<xml_diff>
--- a/data/proteins/pipeline.xlsx
+++ b/data/proteins/pipeline.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB4"/>
+  <dimension ref="A1:AL3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -468,6 +468,16 @@
     <col width="30" customWidth="1" min="26" max="26"/>
     <col width="31" customWidth="1" min="27" max="27"/>
     <col width="34" customWidth="1" min="28" max="28"/>
+    <col width="23" customWidth="1" min="29" max="29"/>
+    <col width="94" customWidth="1" min="30" max="30"/>
+    <col width="102" customWidth="1" min="31" max="31"/>
+    <col width="27" customWidth="1" min="32" max="32"/>
+    <col width="27" customWidth="1" min="33" max="33"/>
+    <col width="27" customWidth="1" min="34" max="34"/>
+    <col width="27" customWidth="1" min="35" max="35"/>
+    <col width="27" customWidth="1" min="36" max="36"/>
+    <col width="27" customWidth="1" min="37" max="37"/>
+    <col width="27" customWidth="1" min="38" max="38"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -611,6 +621,56 @@
           <t>protonation.atom_count_increased</t>
         </is>
       </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>amber_renaming.status</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>amber_renaming.input_path</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>amber_renaming.output_path</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>amber_renaming.his_to_hid</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>amber_renaming.his_to_hie</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>amber_renaming.his_to_hip</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>amber_renaming.asp_to_ash</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>amber_renaming.glu_to_glh</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>amber_renaming.cys_to_cym</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>amber_renaming.cys_to_cyx</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -741,280 +801,242 @@
           <t>True</t>
         </is>
       </c>
+      <c r="AC2" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1IOO/components/1IOO_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1IOO/components/1IOO_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2AFX</t>
+          <t>2P1T</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>33-362</t>
+          <t>229-458</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta/alignments</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta/alignments</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Q16769</t>
+          <t>P19793</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/components</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/components</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta/alignments/filler/A</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta/alignments/filler/A/2P1T_protein_mod.pdb</t>
+        </is>
+      </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>modeller</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta/alignments/filler/A/2P1T_protein_mod.pdb</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/components/2P1T_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>1807</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>3648</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC3" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/components/2P1T_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/components/2P1T_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>6|6</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" s="3" t="inlineStr">
-        <is>
-          <t>warning</t>
-        </is>
-      </c>
-      <c r="P3" s="3" t="inlineStr">
-        <is>
-          <t>warning</t>
-        </is>
-      </c>
-      <c r="Q3" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta/alignments/filler/A</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta/alignments/filler/A/2AFX_protein_mod.pdb</t>
-        </is>
-      </c>
-      <c r="T3" s="3" t="inlineStr">
-        <is>
-          <t>warning</t>
-        </is>
-      </c>
-      <c r="U3" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>modeller</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta/alignments/filler/A/2AFX_protein_mod.pdb</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/components/2AFX_proteinH.pdb</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>7.4</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>2890</t>
-        </is>
-      </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>5726</t>
-        </is>
-      </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2P1T</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>229-458</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta/alignments</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>P19793</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/components</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="P4" s="3" t="inlineStr">
-        <is>
-          <t>warning</t>
-        </is>
-      </c>
-      <c r="Q4" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta/alignments/filler/A</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta/alignments/filler/A/2P1T_protein_mod.pdb</t>
-        </is>
-      </c>
-      <c r="T4" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="U4" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>modeller</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta/alignments/filler/A/2P1T_protein_mod.pdb</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/components/2P1T_proteinH.pdb</t>
-        </is>
-      </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>7.4</t>
-        </is>
-      </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>1807</t>
-        </is>
-      </c>
-      <c r="AA4" t="inlineStr">
-        <is>
-          <t>3648</t>
-        </is>
-      </c>
-      <c r="AB4" t="inlineStr">
-        <is>
-          <t>True</t>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Renumbering od residues to UniProt order
</commit_message>
<xml_diff>
--- a/data/proteins/pipeline.xlsx
+++ b/data/proteins/pipeline.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL3"/>
+  <dimension ref="A1:AT4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -478,6 +478,14 @@
     <col width="27" customWidth="1" min="36" max="36"/>
     <col width="27" customWidth="1" min="37" max="37"/>
     <col width="27" customWidth="1" min="38" max="38"/>
+    <col width="26" customWidth="1" min="39" max="39"/>
+    <col width="102" customWidth="1" min="40" max="40"/>
+    <col width="99" customWidth="1" min="41" max="41"/>
+    <col width="110" customWidth="1" min="42" max="42"/>
+    <col width="26" customWidth="1" min="43" max="43"/>
+    <col width="36" customWidth="1" min="44" max="44"/>
+    <col width="39" customWidth="1" min="45" max="45"/>
+    <col width="82" customWidth="1" min="46" max="46"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -671,6 +679,46 @@
           <t>amber_renaming.cys_to_cyx</t>
         </is>
       </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>numbering_restore.status</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>numbering_restore.input_path</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>numbering_restore.output_path</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>numbering_restore.mapping_path</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>numbering_restore.source</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>numbering_restore.renumbered_atoms</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>numbering_restore.renumbered_residues</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>numbering_restore.message</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -851,194 +899,474 @@
           <t>16</t>
         </is>
       </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>KeyError("Missing finalize numbering entry for chain='B', model_seq_position=1")</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>2AFX</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta/alignments</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Q16769</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/components</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>6|6</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta/alignments/filler/A</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta/alignments/filler/A/2AFX_protein_mod.pdb</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>modeller</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta/alignments/filler/A/2AFX_protein_mod.pdb</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/components/2AFX_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>2890</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>5726</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC3" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/components/2AFX_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/components/2AFX_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/components/2AFX_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AO3" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/components/2AFX_protein_final.pdb</t>
+        </is>
+      </c>
+      <c r="AP3" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta/alignments/2AFX_finalize_numbering.tsv</t>
+        </is>
+      </c>
+      <c r="AQ3" t="inlineStr">
+        <is>
+          <t>finalize_tsv</t>
+        </is>
+      </c>
+      <c r="AR3" t="inlineStr">
+        <is>
+          <t>5726</t>
+        </is>
+      </c>
+      <c r="AS3" t="inlineStr">
+        <is>
+          <t>361</t>
+        </is>
+      </c>
+      <c r="AT3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>2P1T</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>229-458</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta/alignments</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>P19793</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/components</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>warning</t>
         </is>
       </c>
-      <c r="Q3" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
         <is>
           <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta/alignments/filler/A</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta/alignments/filler/A/2P1T_protein_mod.pdb</t>
         </is>
       </c>
-      <c r="T3" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="U3" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="U4" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
         <is>
           <t>modeller</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta/alignments/filler/A/2P1T_protein_mod.pdb</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="X4" t="inlineStr">
         <is>
           <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/components/2P1T_proteinH.pdb</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>7.4</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>1807</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr">
+      <c r="AA4" t="inlineStr">
         <is>
           <t>3648</t>
         </is>
       </c>
-      <c r="AB3" t="inlineStr">
+      <c r="AB4" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="AC3" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="AD3" t="inlineStr">
+      <c r="AC4" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
         <is>
           <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/components/2P1T_proteinH.pdb</t>
         </is>
       </c>
-      <c r="AE3" t="inlineStr">
+      <c r="AE4" t="inlineStr">
         <is>
           <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/components/2P1T_protein_as_Amber.pdb</t>
         </is>
       </c>
-      <c r="AF3" t="inlineStr">
+      <c r="AF4" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="AG3" t="inlineStr">
+      <c r="AG4" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AH3" t="inlineStr">
+      <c r="AH4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AI3" t="inlineStr">
+      <c r="AI4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AJ3" t="inlineStr">
+      <c r="AJ4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AK3" t="inlineStr">
+      <c r="AK4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AL3" t="inlineStr">
+      <c r="AL4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/components/2P1T_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/components/2P1T_protein_final.pdb</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta/alignments/2P1T_finalize_numbering.tsv</t>
+        </is>
+      </c>
+      <c r="AQ4" t="inlineStr">
+        <is>
+          <t>finalize_tsv</t>
+        </is>
+      </c>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>3648</t>
+        </is>
+      </c>
+      <c r="AS4" t="inlineStr">
+        <is>
+          <t>230</t>
+        </is>
+      </c>
+      <c r="AT4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Handling endings and making final model
</commit_message>
<xml_diff>
--- a/data/proteins/pipeline.xlsx
+++ b/data/proteins/pipeline.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT4"/>
+  <dimension ref="A1:AT21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -448,7 +448,7 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="76" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="25" customWidth="1" min="12" max="12"/>
@@ -723,47 +723,47 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1IOO</t>
+          <t>1A5H</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>6-284</t>
+          <t>16-244</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1IOO</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1A5H</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1IOO/fasta</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1A5H/fasta</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1IOO/fasta/alignments</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1A5H/fasta/alignments</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Q7SID5</t>
+          <t>P00750</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1IOO/components</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1A5H/components</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>1|1</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -802,7 +802,11 @@
           <t>success</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr"/>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1A5H/fasta/alignments/filler/A</t>
+        </is>
+      </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" s="2" t="inlineStr">
         <is>
@@ -821,12 +825,12 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1IOO/components/1IOO_protein.pdb</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1A5H/components/1A5H_protein.pdb</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1IOO/components/1IOO_proteinH.pdb</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1A5H/components/1A5H_proteinH.pdb</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -836,12 +840,12 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>3156</t>
+          <t>4844</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>6217</t>
+          <t>7764</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -856,22 +860,22 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1IOO/components/1IOO_proteinH.pdb</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1A5H/components/1A5H_proteinH.pdb</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1IOO/components/1IOO_protein_as_Amber.pdb</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1A5H/components/1A5H_protein_as_Amber.pdb</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>14</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AH2" t="inlineStr">
@@ -896,7 +900,7 @@
       </c>
       <c r="AL2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>20</t>
         </is>
       </c>
       <c r="AM2" t="inlineStr">
@@ -927,43 +931,47 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2AFX</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
+          <t>1B8O</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>3-283</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1B8O</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1B8O/fasta</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta/alignments</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1B8O/fasta/alignments</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Q16769</t>
+          <t>P55859</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/components</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1B8O/components</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>6|6</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1002,19 +1010,11 @@
           <t>success</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta/alignments/filler/A</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta/alignments/filler/A/2AFX_protein_mod.pdb</t>
-        </is>
-      </c>
-      <c r="T3" s="3" t="inlineStr">
-        <is>
-          <t>warning</t>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
@@ -1024,17 +1024,17 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>modeller</t>
+          <t>protein</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta/alignments/filler/A/2AFX_protein_mod.pdb</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1B8O/components/1B8O_protein.pdb</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/components/2AFX_proteinH.pdb</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1B8O/components/1B8O_proteinH.pdb</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
@@ -1044,12 +1044,12 @@
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>2890</t>
+          <t>2199</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>5726</t>
+          <t>4341</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
@@ -1064,37 +1064,37 @@
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/components/2AFX_proteinH.pdb</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1B8O/components/1B8O_proteinH.pdb</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/components/2AFX_protein_as_Amber.pdb</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1B8O/components/1B8O_protein_as_Amber.pdb</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AH3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AI3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AK3" t="inlineStr">
@@ -1114,17 +1114,17 @@
       </c>
       <c r="AN3" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/components/2AFX_protein_as_Amber.pdb</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1B8O/components/1B8O_protein_as_Amber.pdb</t>
         </is>
       </c>
       <c r="AO3" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/components/2AFX_protein_final.pdb</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1B8O/components/1B8O_protein_final.pdb</t>
         </is>
       </c>
       <c r="AP3" t="inlineStr">
         <is>
-          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta/alignments/2AFX_finalize_numbering.tsv</t>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1B8O/fasta/alignments/1B8O_finalize_numbering.tsv</t>
         </is>
       </c>
       <c r="AQ3" t="inlineStr">
@@ -1134,12 +1134,12 @@
       </c>
       <c r="AR3" t="inlineStr">
         <is>
-          <t>5726</t>
+          <t>4341</t>
         </is>
       </c>
       <c r="AS3" t="inlineStr">
         <is>
-          <t>361</t>
+          <t>280</t>
         </is>
       </c>
       <c r="AT3" t="inlineStr"/>
@@ -1147,226 +1147,3858 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>1F0R</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>16-50</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1F0R</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1F0R/fasta</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1F0R/fasta/alignments</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>P00742</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1F0R/components</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="U4" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>protein</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1F0R/components/1F0R_protein.pdb</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1F0R/components/1F0R_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>1002</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC4" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1F0R/components/1F0R_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1F0R/components/1F0R_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="AN4" t="inlineStr"/>
+      <c r="AO4" t="inlineStr"/>
+      <c r="AP4" t="inlineStr"/>
+      <c r="AQ4" t="inlineStr"/>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AS4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AT4" t="inlineStr">
+        <is>
+          <t>KeyError("Missing finalize numbering entry for chain='B', model_seq_position=1")</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1I00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>6-306</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1I00</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1I00/fasta</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1I00/fasta/alignments</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>P04818</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1I00/components</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>23|23</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P5" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1I00/fasta/alignments/filler/A</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="U5" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>protein</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1I00/components/1I00_protein.pdb</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1I00/components/1I00_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>4520</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>8936</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC5" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1I00/components/1I00_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1I00/components/1I00_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr"/>
+      <c r="AO5" t="inlineStr"/>
+      <c r="AP5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr"/>
+      <c r="AR5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AS5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AT5" t="inlineStr">
+        <is>
+          <t>KeyError("Missing finalize numbering entry for chain='B', model_seq_position=1")</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1UOU</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>33-480</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1UOU</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1UOU/fasta</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1UOU/fasta/alignments</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>P19971</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1UOU/components</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2|8</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P6" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1UOU/fasta/alignments/filler/A</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1UOU/fasta/alignments/filler/A/1UOU_protein_mod.pdb</t>
+        </is>
+      </c>
+      <c r="T6" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="U6" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>modeller</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1UOU/fasta/alignments/filler/A/1UOU_protein_mod.pdb</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1UOU/components/1UOU_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>3502</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>7084</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC6" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1UOU/components/1UOU_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1UOU/components/1UOU_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1UOU/components/1UOU_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1UOU/components/1UOU_protein_final.pdb</t>
+        </is>
+      </c>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1UOU/fasta/alignments/1UOU_finalize_numbering.tsv</t>
+        </is>
+      </c>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>finalize_tsv</t>
+        </is>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>7084</t>
+        </is>
+      </c>
+      <c r="AS6" t="inlineStr">
+        <is>
+          <t>482</t>
+        </is>
+      </c>
+      <c r="AT6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1W4R</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>18-191</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1W4R</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1W4R/fasta</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1W4R/fasta/alignments</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>P04183</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1W4R/components</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>7|14|14|14|13|14|13</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="P7" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1W4R/fasta/alignments/filler/A</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="U7" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>protein</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1W4R/components/1W4R_protein.pdb</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1W4R/components/1W4R_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>10203</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>20578</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC7" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1W4R/components/1W4R_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/1W4R/components/1W4R_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="AN7" t="inlineStr"/>
+      <c r="AO7" t="inlineStr"/>
+      <c r="AP7" t="inlineStr"/>
+      <c r="AQ7" t="inlineStr"/>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AS7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AT7" t="inlineStr">
+        <is>
+          <t>KeyError("Missing finalize numbering entry for chain='B', model_seq_position=1")</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2AFX</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>33-361</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta/alignments</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Q16769</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/components</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>6|6</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta/alignments/filler/A</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta/alignments/filler/A/2AFX_protein_mod.pdb</t>
+        </is>
+      </c>
+      <c r="T8" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="U8" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>modeller</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta/alignments/filler/A/2AFX_protein_mod.pdb</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/components/2AFX_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>2890</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>5726</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC8" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/components/2AFX_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/components/2AFX_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AK8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AM8" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AN8" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/components/2AFX_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/components/2AFX_protein_final.pdb</t>
+        </is>
+      </c>
+      <c r="AP8" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2AFX/fasta/alignments/2AFX_finalize_numbering.tsv</t>
+        </is>
+      </c>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>finalize_tsv</t>
+        </is>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>5726</t>
+        </is>
+      </c>
+      <c r="AS8" t="inlineStr">
+        <is>
+          <t>361</t>
+        </is>
+      </c>
+      <c r="AT8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>2P1T</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>229-458</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta/alignments</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>P19793</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/components</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P9" s="3" t="inlineStr">
         <is>
           <t>warning</t>
         </is>
       </c>
-      <c r="Q4" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
         <is>
           <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta/alignments/filler/A</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta/alignments/filler/A/2P1T_protein_mod.pdb</t>
         </is>
       </c>
-      <c r="T4" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="U4" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
+      <c r="T9" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="U9" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
         <is>
           <t>modeller</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="W9" t="inlineStr">
         <is>
           <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta/alignments/filler/A/2P1T_protein_mod.pdb</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="X9" t="inlineStr">
         <is>
           <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/components/2P1T_proteinH.pdb</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr">
+      <c r="Y9" t="inlineStr">
         <is>
           <t>7.4</t>
         </is>
       </c>
-      <c r="Z4" t="inlineStr">
+      <c r="Z9" t="inlineStr">
         <is>
           <t>1807</t>
         </is>
       </c>
-      <c r="AA4" t="inlineStr">
+      <c r="AA9" t="inlineStr">
         <is>
           <t>3648</t>
         </is>
       </c>
-      <c r="AB4" t="inlineStr">
+      <c r="AB9" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="AC4" s="2" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="AD4" t="inlineStr">
+      <c r="AC9" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
         <is>
           <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/components/2P1T_proteinH.pdb</t>
         </is>
       </c>
-      <c r="AE4" t="inlineStr">
+      <c r="AE9" t="inlineStr">
         <is>
           <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/components/2P1T_protein_as_Amber.pdb</t>
         </is>
       </c>
-      <c r="AF4" t="inlineStr">
+      <c r="AF9" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="AG4" t="inlineStr">
+      <c r="AG9" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AH4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AI4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AJ4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AK4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AL4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AM4" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="AN4" t="inlineStr">
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AN9" t="inlineStr">
         <is>
           <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/components/2P1T_protein_as_Amber.pdb</t>
         </is>
       </c>
-      <c r="AO4" t="inlineStr">
+      <c r="AO9" t="inlineStr">
         <is>
           <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/components/2P1T_protein_final.pdb</t>
         </is>
       </c>
-      <c r="AP4" t="inlineStr">
+      <c r="AP9" t="inlineStr">
         <is>
           <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2P1T/fasta/alignments/2P1T_finalize_numbering.tsv</t>
         </is>
       </c>
-      <c r="AQ4" t="inlineStr">
+      <c r="AQ9" t="inlineStr">
         <is>
           <t>finalize_tsv</t>
         </is>
       </c>
-      <c r="AR4" t="inlineStr">
+      <c r="AR9" t="inlineStr">
         <is>
           <t>3648</t>
         </is>
       </c>
-      <c r="AS4" t="inlineStr">
+      <c r="AS9" t="inlineStr">
         <is>
           <t>230</t>
         </is>
       </c>
-      <c r="AT4" t="inlineStr"/>
+      <c r="AT9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2W8Y</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>683-932</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2W8Y</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2W8Y/fasta</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2W8Y/fasta/alignments</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>P06401</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2W8Y/components</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P10" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>protein</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2W8Y/components/2W8Y_protein.pdb</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2W8Y/components/2W8Y_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>4105</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>8242</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC10" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2W8Y/components/2W8Y_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2W8Y/components/2W8Y_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="AN10" t="inlineStr"/>
+      <c r="AO10" t="inlineStr"/>
+      <c r="AP10" t="inlineStr"/>
+      <c r="AQ10" t="inlineStr"/>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AS10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AT10" t="inlineStr">
+        <is>
+          <t>KeyError("Missing finalize numbering entry for chain='B', model_seq_position=1")</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2WCG</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0-497</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2WCG</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2WCG/fasta</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2WCG/fasta/alignments</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>P04062</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2WCG/components</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>5|3</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P11" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2WCG/fasta/alignments/filler/A</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2WCG/fasta/alignments/filler/A/2WCG_protein_mod.pdb</t>
+        </is>
+      </c>
+      <c r="T11" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>modeller</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2WCG/fasta/alignments/filler/A/2WCG_protein_mod.pdb</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2WCG/components/2WCG_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>4218</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>8364</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC11" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2WCG/components/2WCG_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2WCG/components/2WCG_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AH11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AI11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AK11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL11" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AM11" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AN11" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2WCG/components/2WCG_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AO11" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2WCG/components/2WCG_protein_final.pdb</t>
+        </is>
+      </c>
+      <c r="AP11" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/2WCG/fasta/alignments/2WCG_finalize_numbering.tsv</t>
+        </is>
+      </c>
+      <c r="AQ11" t="inlineStr">
+        <is>
+          <t>finalize_tsv</t>
+        </is>
+      </c>
+      <c r="AR11" t="inlineStr">
+        <is>
+          <t>8364</t>
+        </is>
+      </c>
+      <c r="AS11" t="inlineStr">
+        <is>
+          <t>536</t>
+        </is>
+      </c>
+      <c r="AT11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>3BC3</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1-220</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3BC3</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3BC3/fasta</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3BC3/fasta/alignments</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>P07711</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3BC3/components</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>5|5</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P12" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>protein</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3BC3/components/3BC3_protein.pdb</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3BC3/components/3BC3_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>3322</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>6388</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC12" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3BC3/components/3BC3_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3BC3/components/3BC3_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AH12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AK12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL12" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="AM12" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="AN12" t="inlineStr"/>
+      <c r="AO12" t="inlineStr"/>
+      <c r="AP12" t="inlineStr"/>
+      <c r="AQ12" t="inlineStr"/>
+      <c r="AR12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AS12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AT12" t="inlineStr">
+        <is>
+          <t>KeyError("Missing finalize numbering entry for chain='B', model_seq_position=1")</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>3EWJ</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>220-474</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3EWJ</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3EWJ/fasta</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3EWJ/fasta/alignments</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>P78536</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3EWJ/components</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="P13" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3EWJ/fasta/alignments/filler/A</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3EWJ/fasta/alignments/filler/A/3EWJ_protein_mod.pdb</t>
+        </is>
+      </c>
+      <c r="T13" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>modeller</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3EWJ/fasta/alignments/filler/A/3EWJ_protein_mod.pdb</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3EWJ/components/3EWJ_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>6517</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>12847</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC13" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3EWJ/components/3EWJ_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3EWJ/components/3EWJ_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AI13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AK13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL13" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AM13" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AN13" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3EWJ/components/3EWJ_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AO13" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3EWJ/components/3EWJ_protein_final.pdb</t>
+        </is>
+      </c>
+      <c r="AP13" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3EWJ/fasta/alignments/3EWJ_finalize_numbering.tsv</t>
+        </is>
+      </c>
+      <c r="AQ13" t="inlineStr">
+        <is>
+          <t>finalize_tsv</t>
+        </is>
+      </c>
+      <c r="AR13" t="inlineStr">
+        <is>
+          <t>12847</t>
+        </is>
+      </c>
+      <c r="AS13" t="inlineStr">
+        <is>
+          <t>824</t>
+        </is>
+      </c>
+      <c r="AT13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>3FDN</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>126-394</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3FDN</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3FDN/fasta</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3FDN/fasta/alignments</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>O14965</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3FDN/components</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P14" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3FDN/fasta/alignments/filler/A</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3FDN/fasta/alignments/filler/A/3FDN_protein_mod.pdb</t>
+        </is>
+      </c>
+      <c r="T14" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>modeller</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3FDN/fasta/alignments/filler/A/3FDN_protein_mod.pdb</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3FDN/components/3FDN_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>3229</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>6493</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC14" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3FDN/components/3FDN_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3FDN/components/3FDN_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AG14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AI14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AJ14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AK14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AM14" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AN14" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3FDN/components/3FDN_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AO14" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3FDN/components/3FDN_protein_final.pdb</t>
+        </is>
+      </c>
+      <c r="AP14" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3FDN/fasta/alignments/3FDN_finalize_numbering.tsv</t>
+        </is>
+      </c>
+      <c r="AQ14" t="inlineStr">
+        <is>
+          <t>finalize_tsv</t>
+        </is>
+      </c>
+      <c r="AR14" t="inlineStr">
+        <is>
+          <t>6493</t>
+        </is>
+      </c>
+      <c r="AS14" t="inlineStr">
+        <is>
+          <t>403</t>
+        </is>
+      </c>
+      <c r="AT14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>3FRG</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>153-487</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3FRG</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3FRG/fasta</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3FRG/fasta/alignments</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Q07343</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3FRG/components</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="P15" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>protein</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3FRG/components/3FRG_protein.pdb</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3FRG/components/3FRG_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>2708</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>5344</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC15" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3FRG/components/3FRG_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3FRG/components/3FRG_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AH15" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AI15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AJ15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AM15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AN15" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3FRG/components/3FRG_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AO15" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3FRG/components/3FRG_protein_final.pdb</t>
+        </is>
+      </c>
+      <c r="AP15" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3FRG/fasta/alignments/3FRG_finalize_numbering.tsv</t>
+        </is>
+      </c>
+      <c r="AQ15" t="inlineStr">
+        <is>
+          <t>finalize_tsv</t>
+        </is>
+      </c>
+      <c r="AR15" t="inlineStr">
+        <is>
+          <t>5344</t>
+        </is>
+      </c>
+      <c r="AS15" t="inlineStr">
+        <is>
+          <t>335</t>
+        </is>
+      </c>
+      <c r="AT15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>3K5E</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>18-364</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3K5E</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3K5E/fasta</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3K5E/fasta/alignments</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>P52732</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3K5E/components</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2|15|1|2|3|15</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="P16" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3K5E/fasta/alignments/filler/A</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3K5E/fasta/alignments/filler/A/3K5E_protein_mod.pdb</t>
+        </is>
+      </c>
+      <c r="T16" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>modeller</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3K5E/fasta/alignments/filler/A/3K5E_protein_mod.pdb</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3K5E/components/3K5E_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>2717</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>5464</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC16" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3K5E/components/3K5E_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3K5E/components/3K5E_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AH16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AJ16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AM16" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AN16" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3K5E/components/3K5E_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AO16" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3K5E/components/3K5E_protein_final.pdb</t>
+        </is>
+      </c>
+      <c r="AP16" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3K5E/fasta/alignments/3K5E_finalize_numbering.tsv</t>
+        </is>
+      </c>
+      <c r="AQ16" t="inlineStr">
+        <is>
+          <t>finalize_tsv</t>
+        </is>
+      </c>
+      <c r="AR16" t="inlineStr">
+        <is>
+          <t>5464</t>
+        </is>
+      </c>
+      <c r="AS16" t="inlineStr">
+        <is>
+          <t>347</t>
+        </is>
+      </c>
+      <c r="AT16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>3L3M</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2-349</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3L3M</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3L3M/fasta</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3L3M/fasta/alignments</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>P09874</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3L3M/components</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P17" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>protein</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3L3M/components/3L3M_protein.pdb</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3L3M/components/3L3M_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>2735</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>5510</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC17" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3L3M/components/3L3M_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3L3M/components/3L3M_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AH17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AJ17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AM17" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AN17" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3L3M/components/3L3M_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AO17" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3L3M/components/3L3M_protein_final.pdb</t>
+        </is>
+      </c>
+      <c r="AP17" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3L3M/fasta/alignments/3L3M_finalize_numbering.tsv</t>
+        </is>
+      </c>
+      <c r="AQ17" t="inlineStr">
+        <is>
+          <t>finalize_tsv</t>
+        </is>
+      </c>
+      <c r="AR17" t="inlineStr">
+        <is>
+          <t>5510</t>
+        </is>
+      </c>
+      <c r="AS17" t="inlineStr">
+        <is>
+          <t>348</t>
+        </is>
+      </c>
+      <c r="AT17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>3LBK</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>26-110</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3LBK</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3LBK/fasta</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3LBK/fasta/alignments</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Q00987</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3LBK/components</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P18" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="Q18" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="U18" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>protein</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3LBK/components/3LBK_protein.pdb</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3LBK/components/3LBK_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>695</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>1446</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC18" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3LBK/components/3LBK_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3LBK/components/3LBK_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AH18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AJ18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AM18" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AN18" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3LBK/components/3LBK_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AO18" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3LBK/components/3LBK_protein_final.pdb</t>
+        </is>
+      </c>
+      <c r="AP18" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3LBK/fasta/alignments/3LBK_finalize_numbering.tsv</t>
+        </is>
+      </c>
+      <c r="AQ18" t="inlineStr">
+        <is>
+          <t>finalize_tsv</t>
+        </is>
+      </c>
+      <c r="AR18" t="inlineStr">
+        <is>
+          <t>1446</t>
+        </is>
+      </c>
+      <c r="AS18" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="AT18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>3OLL</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>262-498</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3OLL</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3OLL/fasta</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3OLL/fasta/alignments</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Q15788</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3OLL/components</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2|3</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P19" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="Q19" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>protein</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3OLL/components/3OLL_protein.pdb</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3OLL/components/3OLL_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>3787</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>7511</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC19" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3OLL/components/3OLL_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3OLL/components/3OLL_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AH19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AJ19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AK19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AM19" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="AN19" t="inlineStr"/>
+      <c r="AO19" t="inlineStr"/>
+      <c r="AP19" t="inlineStr"/>
+      <c r="AQ19" t="inlineStr"/>
+      <c r="AR19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AS19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AT19" t="inlineStr">
+        <is>
+          <t>KeyError("Missing finalize numbering entry for chain='B', model_seq_position=1")</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>3R04</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>35-305</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3R04</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3R04/fasta</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3R04/fasta/alignments</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>P11309</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3R04/components</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="P20" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="Q20" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="U20" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>protein</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3R04/components/3R04_protein.pdb</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3R04/components/3R04_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>2225</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>4365</t>
+        </is>
+      </c>
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC20" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3R04/components/3R04_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3R04/components/3R04_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AG20" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AH20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AJ20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AM20" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AN20" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3R04/components/3R04_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AO20" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3R04/components/3R04_protein_final.pdb</t>
+        </is>
+      </c>
+      <c r="AP20" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3R04/fasta/alignments/3R04_finalize_numbering.tsv</t>
+        </is>
+      </c>
+      <c r="AQ20" t="inlineStr">
+        <is>
+          <t>finalize_tsv</t>
+        </is>
+      </c>
+      <c r="AR20" t="inlineStr">
+        <is>
+          <t>4365</t>
+        </is>
+      </c>
+      <c r="AS20" t="inlineStr">
+        <is>
+          <t>271</t>
+        </is>
+      </c>
+      <c r="AT20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>3RM2</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>16-246</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3RM2</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3RM2/fasta</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3RM2/fasta/alignments</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>P00734</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3RM2/components</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2|1|1</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="P21" s="3" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="Q21" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>protein</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3RM2/components/3RM2_protein.pdb</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3RM2/components/3RM2_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>2163</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>4203</t>
+        </is>
+      </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC21" s="2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3RM2/components/3RM2_proteinH.pdb</t>
+        </is>
+      </c>
+      <c r="AE21" t="inlineStr">
+        <is>
+          <t>/home/grheco/repositorios/stack_protein_prep/data/proteins/3RM2/components/3RM2_protein_as_Amber.pdb</t>
+        </is>
+      </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AH21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AJ21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL21" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AM21" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="AN21" t="inlineStr"/>
+      <c r="AO21" t="inlineStr"/>
+      <c r="AP21" t="inlineStr"/>
+      <c r="AQ21" t="inlineStr"/>
+      <c r="AR21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AS21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AT21" t="inlineStr">
+        <is>
+          <t>KeyError("Missing finalize numbering entry for chain='I', model_seq_position=1")</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: regenerate prepared structures with unique chain IDs per gap fragment
Re-run FRUTON after fixing prepared_structure.py to assign sequential
chain IDs (A, B, C, …) to gap fragments on merge.  The previous output
had all fragments on chain A, causing BioPython to collapse them into a
single chain and strip internal TER records.  pdb2gmx then saw internal
capped C-termini as regular residues and failed with "Atom OC1 not found
in rtp entry LYS".

Six gaps variants now pass the parameter audit (2AFX, 2P1T, 3BC3, 3K5E,
3OLL gaps; 3RM2).  Remaining rejections are metals-policy, not topology.
</commit_message>
<xml_diff>
--- a/data/proteins/pipeline.xlsx
+++ b/data/proteins/pipeline.xlsx
@@ -21,10 +21,10 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'preparation'!$A$1:$G$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'components'!$A$1:$I$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'gaps_and_variants'!$A$1:$L$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'chemistry'!$A$1:$L$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'prepared_outputs'!$A$1:$L$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'paths'!$A$1:$P$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'full_state'!$A$1:$AY$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'chemistry'!$A$1:$M$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'prepared_outputs'!$A$1:$M$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'paths'!$A$1:$Q$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'full_state'!$A$1:$BB$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -754,7 +754,7 @@
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="D4" s="9" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="F4" s="10" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
@@ -1487,12 +1487,12 @@
       </c>
       <c r="E14" s="17" t="inlineStr">
         <is>
-          <t>large_gap_complete</t>
+          <t>gaps,large_gap_complete</t>
         </is>
       </c>
       <c r="F14" s="17" t="inlineStr">
         <is>
-          <t>alphafold</t>
+          <t>gaps | alphafold</t>
         </is>
       </c>
       <c r="G14" s="17" t="inlineStr">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="O14" s="17" t="inlineStr">
         <is>
-          <t>large_gap_complete</t>
+          <t>gaps,large_gap_complete</t>
         </is>
       </c>
     </row>
@@ -1706,12 +1706,12 @@
       </c>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>best_complete</t>
+          <t>gaps,best_complete</t>
         </is>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>modeller</t>
+          <t>gaps | modeller</t>
         </is>
       </c>
       <c r="G17" s="13" t="inlineStr">
@@ -1756,7 +1756,7 @@
       </c>
       <c r="O17" s="13" t="inlineStr">
         <is>
-          <t>best_complete</t>
+          <t>gaps,best_complete</t>
         </is>
       </c>
     </row>
@@ -1968,7 +1968,7 @@
       <c r="O20" s="17" t="inlineStr"/>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="21" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>3K5E</t>
         </is>
@@ -1983,13 +1983,21 @@
           <t>18-363</t>
         </is>
       </c>
-      <c r="D21" s="21" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="E21" s="13" t="inlineStr"/>
-      <c r="F21" s="13" t="inlineStr"/>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E21" s="13" t="inlineStr">
+        <is>
+          <t>gaps</t>
+        </is>
+      </c>
+      <c r="F21" s="13" t="inlineStr">
+        <is>
+          <t>gaps</t>
+        </is>
+      </c>
       <c r="G21" s="18" t="inlineStr">
         <is>
           <t>yes</t>
@@ -2025,12 +2033,16 @@
           <t>skipped</t>
         </is>
       </c>
-      <c r="N21" s="20" t="inlineStr">
-        <is>
-          <t>failed</t>
-        </is>
-      </c>
-      <c r="O21" s="13" t="inlineStr"/>
+      <c r="N21" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="O21" s="13" t="inlineStr">
+        <is>
+          <t>gaps</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="16" t="inlineStr">
@@ -2197,12 +2209,12 @@
       </c>
       <c r="E24" s="17" t="inlineStr">
         <is>
-          <t>best_complete</t>
+          <t>gaps,best_complete</t>
         </is>
       </c>
       <c r="F24" s="17" t="inlineStr">
         <is>
-          <t>alphafold</t>
+          <t>gaps | alphafold</t>
         </is>
       </c>
       <c r="G24" s="17" t="inlineStr">
@@ -2247,7 +2259,7 @@
       </c>
       <c r="O24" s="17" t="inlineStr">
         <is>
-          <t>best_complete</t>
+          <t>gaps,best_complete</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2956,7 @@
       <c r="G15" s="17" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>3K5E</t>
         </is>
@@ -3877,7 +3889,7 @@
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>3K5E</t>
         </is>
@@ -4696,12 +4708,12 @@
       </c>
       <c r="K9" s="17" t="inlineStr">
         <is>
-          <t>large_gap_complete</t>
+          <t>gaps,large_gap_complete</t>
         </is>
       </c>
       <c r="L9" s="17" t="inlineStr">
         <is>
-          <t>alphafold</t>
+          <t>gaps | alphafold</t>
         </is>
       </c>
     </row>
@@ -4870,12 +4882,12 @@
       </c>
       <c r="K12" s="13" t="inlineStr">
         <is>
-          <t>best_complete</t>
+          <t>gaps,best_complete</t>
         </is>
       </c>
       <c r="L12" s="13" t="inlineStr">
         <is>
-          <t>modeller</t>
+          <t>gaps | modeller</t>
         </is>
       </c>
     </row>
@@ -5042,7 +5054,7 @@
       <c r="L15" s="17" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>3K5E</t>
         </is>
@@ -5088,8 +5100,16 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K16" s="13" t="inlineStr"/>
-      <c r="L16" s="13" t="inlineStr"/>
+      <c r="K16" s="13" t="inlineStr">
+        <is>
+          <t>gaps</t>
+        </is>
+      </c>
+      <c r="L16" s="13" t="inlineStr">
+        <is>
+          <t>gaps</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
@@ -5252,12 +5272,12 @@
       </c>
       <c r="K19" s="17" t="inlineStr">
         <is>
-          <t>best_complete</t>
+          <t>gaps,best_complete</t>
         </is>
       </c>
       <c r="L19" s="17" t="inlineStr">
         <is>
-          <t>alphafold</t>
+          <t>gaps | alphafold</t>
         </is>
       </c>
     </row>
@@ -5381,7 +5401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5396,6 +5416,7 @@
     <col width="28" customWidth="1" min="10" max="10"/>
     <col width="28" customWidth="1" min="11" max="11"/>
     <col width="23" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5459,6 +5480,11 @@
           <t>metals.geometry_match</t>
         </is>
       </c>
+      <c r="M1" s="12" t="inlineStr">
+        <is>
+          <t>metall_params.status</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="8" t="inlineStr">
@@ -5521,6 +5547,7 @@
           <t>n/a</t>
         </is>
       </c>
+      <c r="M2" s="13" t="inlineStr"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="16" t="inlineStr">
@@ -5583,6 +5610,11 @@
           <t>n/a</t>
         </is>
       </c>
+      <c r="M3" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -5645,6 +5677,11 @@
           <t>n/a</t>
         </is>
       </c>
+      <c r="M4" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="16" t="inlineStr">
@@ -5707,6 +5744,7 @@
           <t>n/a</t>
         </is>
       </c>
+      <c r="M5" s="17" t="inlineStr"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -5769,6 +5807,7 @@
           <t>n/a</t>
         </is>
       </c>
+      <c r="M6" s="13" t="inlineStr"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="19" t="inlineStr">
@@ -5831,6 +5870,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="M7" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="21" t="inlineStr">
@@ -5893,6 +5937,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="M8" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="16" t="inlineStr">
@@ -5955,6 +6004,7 @@
           <t>n/a</t>
         </is>
       </c>
+      <c r="M9" s="17" t="inlineStr"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="21" t="inlineStr">
@@ -6017,6 +6067,7 @@
           <t>n/a</t>
         </is>
       </c>
+      <c r="M10" s="13" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="16" t="inlineStr">
@@ -6079,6 +6130,7 @@
           <t>n/a</t>
         </is>
       </c>
+      <c r="M11" s="17" t="inlineStr"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -6141,6 +6193,7 @@
           <t>n/a</t>
         </is>
       </c>
+      <c r="M12" s="13" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="19" t="inlineStr">
@@ -6203,6 +6256,11 @@
           <t>no</t>
         </is>
       </c>
+      <c r="M13" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -6265,6 +6323,7 @@
           <t>n/a</t>
         </is>
       </c>
+      <c r="M14" s="13" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="19" t="inlineStr">
@@ -6327,9 +6386,14 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="M15" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>3K5E</t>
         </is>
@@ -6387,6 +6451,11 @@
       <c r="L16" s="22" t="inlineStr">
         <is>
           <t>n/a</t>
+        </is>
+      </c>
+      <c r="M16" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
         </is>
       </c>
     </row>
@@ -6451,6 +6520,7 @@
           <t>n/a</t>
         </is>
       </c>
+      <c r="M17" s="17" t="inlineStr"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="21" t="inlineStr">
@@ -6513,6 +6583,7 @@
           <t>n/a</t>
         </is>
       </c>
+      <c r="M18" s="13" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
@@ -6575,6 +6646,7 @@
           <t>n/a</t>
         </is>
       </c>
+      <c r="M19" s="17" t="inlineStr"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -6637,6 +6709,7 @@
           <t>n/a</t>
         </is>
       </c>
+      <c r="M20" s="13" t="inlineStr"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="19" t="inlineStr">
@@ -6699,9 +6772,14 @@
           <t>n/a</t>
         </is>
       </c>
+      <c r="M21" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L21"/>
+  <autoFilter ref="A1:M21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6712,12 +6790,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
@@ -6727,6 +6805,7 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6782,10 +6861,15 @@
       </c>
       <c r="K1" s="12" t="inlineStr">
         <is>
+          <t>prepared.gaps.output_path</t>
+        </is>
+      </c>
+      <c r="L1" s="12" t="inlineStr">
+        <is>
           <t>prepared.modeller.output_path</t>
         </is>
       </c>
-      <c r="L1" s="12" t="inlineStr">
+      <c r="M1" s="12" t="inlineStr">
         <is>
           <t>prepared.alphafold.output_path</t>
         </is>
@@ -6844,6 +6928,7 @@
       </c>
       <c r="K2" s="13" t="inlineStr"/>
       <c r="L2" s="13" t="inlineStr"/>
+      <c r="M2" s="13" t="inlineStr"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="16" t="inlineStr">
@@ -6898,6 +6983,7 @@
       </c>
       <c r="K3" s="17" t="inlineStr"/>
       <c r="L3" s="17" t="inlineStr"/>
+      <c r="M3" s="17" t="inlineStr"/>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -6952,6 +7038,7 @@
       </c>
       <c r="K4" s="13" t="inlineStr"/>
       <c r="L4" s="13" t="inlineStr"/>
+      <c r="M4" s="13" t="inlineStr"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="16" t="inlineStr">
@@ -7006,6 +7093,7 @@
       </c>
       <c r="K5" s="17" t="inlineStr"/>
       <c r="L5" s="17" t="inlineStr"/>
+      <c r="M5" s="17" t="inlineStr"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -7059,7 +7147,8 @@
         </is>
       </c>
       <c r="K6" s="13" t="inlineStr"/>
-      <c r="L6" s="29" t="inlineStr">
+      <c r="L6" s="13" t="inlineStr"/>
+      <c r="M6" s="29" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -7098,6 +7187,7 @@
       <c r="J7" s="17" t="inlineStr"/>
       <c r="K7" s="17" t="inlineStr"/>
       <c r="L7" s="17" t="inlineStr"/>
+      <c r="M7" s="17" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="21" t="inlineStr">
@@ -7132,6 +7222,7 @@
       <c r="J8" s="13" t="inlineStr"/>
       <c r="K8" s="13" t="inlineStr"/>
       <c r="L8" s="13" t="inlineStr"/>
+      <c r="M8" s="13" t="inlineStr"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="16" t="inlineStr">
@@ -7146,12 +7237,12 @@
       </c>
       <c r="C9" s="17" t="inlineStr">
         <is>
-          <t>large_gap_complete</t>
+          <t>gaps,large_gap_complete</t>
         </is>
       </c>
       <c r="D9" s="17" t="inlineStr">
         <is>
-          <t>alphafold</t>
+          <t>gaps | alphafold</t>
         </is>
       </c>
       <c r="E9" s="17" t="inlineStr">
@@ -7171,7 +7262,7 @@
       </c>
       <c r="H9" s="17" t="inlineStr">
         <is>
-          <t>large_gap_complete</t>
+          <t>gaps,large_gap_complete</t>
         </is>
       </c>
       <c r="I9" s="30" t="inlineStr">
@@ -7184,8 +7275,13 @@
           <t>open</t>
         </is>
       </c>
-      <c r="K9" s="17" t="inlineStr"/>
-      <c r="L9" s="30" t="inlineStr">
+      <c r="K9" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="L9" s="17" t="inlineStr"/>
+      <c r="M9" s="30" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -7224,6 +7320,7 @@
       <c r="J10" s="13" t="inlineStr"/>
       <c r="K10" s="13" t="inlineStr"/>
       <c r="L10" s="13" t="inlineStr"/>
+      <c r="M10" s="13" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="16" t="inlineStr">
@@ -7277,7 +7374,8 @@
         </is>
       </c>
       <c r="K11" s="17" t="inlineStr"/>
-      <c r="L11" s="30" t="inlineStr">
+      <c r="L11" s="17" t="inlineStr"/>
+      <c r="M11" s="30" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -7296,12 +7394,12 @@
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>best_complete</t>
+          <t>gaps,best_complete</t>
         </is>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>modeller</t>
+          <t>gaps | modeller</t>
         </is>
       </c>
       <c r="E12" s="13" t="inlineStr">
@@ -7321,7 +7419,7 @@
       </c>
       <c r="H12" s="13" t="inlineStr">
         <is>
-          <t>best_complete</t>
+          <t>gaps,best_complete</t>
         </is>
       </c>
       <c r="I12" s="29" t="inlineStr">
@@ -7339,7 +7437,12 @@
           <t>open</t>
         </is>
       </c>
-      <c r="L12" s="13" t="inlineStr"/>
+      <c r="L12" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="M12" s="13" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="19" t="inlineStr">
@@ -7374,6 +7477,7 @@
       <c r="J13" s="17" t="inlineStr"/>
       <c r="K13" s="17" t="inlineStr"/>
       <c r="L13" s="17" t="inlineStr"/>
+      <c r="M13" s="17" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -7427,7 +7531,8 @@
         </is>
       </c>
       <c r="K14" s="13" t="inlineStr"/>
-      <c r="L14" s="29" t="inlineStr">
+      <c r="L14" s="13" t="inlineStr"/>
+      <c r="M14" s="29" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -7466,20 +7571,29 @@
       <c r="J15" s="17" t="inlineStr"/>
       <c r="K15" s="17" t="inlineStr"/>
       <c r="L15" s="17" t="inlineStr"/>
+      <c r="M15" s="17" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>3K5E</t>
         </is>
       </c>
-      <c r="B16" s="21" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="C16" s="13" t="inlineStr"/>
-      <c r="D16" s="13" t="inlineStr"/>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>gaps</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>gaps</t>
+        </is>
+      </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
           <t>yes</t>
@@ -7490,16 +7604,33 @@
           <t>success</t>
         </is>
       </c>
-      <c r="G16" s="20" t="inlineStr">
-        <is>
-          <t>failed</t>
-        </is>
-      </c>
-      <c r="H16" s="13" t="inlineStr"/>
-      <c r="I16" s="13" t="inlineStr"/>
-      <c r="J16" s="13" t="inlineStr"/>
-      <c r="K16" s="13" t="inlineStr"/>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="H16" s="13" t="inlineStr">
+        <is>
+          <t>gaps</t>
+        </is>
+      </c>
+      <c r="I16" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="J16" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="K16" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="L16" s="13" t="inlineStr"/>
+      <c r="M16" s="13" t="inlineStr"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
@@ -7554,6 +7685,7 @@
       </c>
       <c r="K17" s="17" t="inlineStr"/>
       <c r="L17" s="17" t="inlineStr"/>
+      <c r="M17" s="17" t="inlineStr"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="21" t="inlineStr">
@@ -7588,6 +7720,7 @@
       <c r="J18" s="13" t="inlineStr"/>
       <c r="K18" s="13" t="inlineStr"/>
       <c r="L18" s="13" t="inlineStr"/>
+      <c r="M18" s="13" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
@@ -7602,12 +7735,12 @@
       </c>
       <c r="C19" s="17" t="inlineStr">
         <is>
-          <t>best_complete</t>
+          <t>gaps,best_complete</t>
         </is>
       </c>
       <c r="D19" s="17" t="inlineStr">
         <is>
-          <t>alphafold</t>
+          <t>gaps | alphafold</t>
         </is>
       </c>
       <c r="E19" s="17" t="inlineStr">
@@ -7627,7 +7760,7 @@
       </c>
       <c r="H19" s="17" t="inlineStr">
         <is>
-          <t>best_complete</t>
+          <t>gaps,best_complete</t>
         </is>
       </c>
       <c r="I19" s="30" t="inlineStr">
@@ -7640,8 +7773,13 @@
           <t>open</t>
         </is>
       </c>
-      <c r="K19" s="17" t="inlineStr"/>
-      <c r="L19" s="30" t="inlineStr">
+      <c r="K19" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="L19" s="17" t="inlineStr"/>
+      <c r="M19" s="30" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -7700,6 +7838,7 @@
       </c>
       <c r="K20" s="13" t="inlineStr"/>
       <c r="L20" s="13" t="inlineStr"/>
+      <c r="M20" s="13" t="inlineStr"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="19" t="inlineStr">
@@ -7734,9 +7873,10 @@
       <c r="J21" s="17" t="inlineStr"/>
       <c r="K21" s="17" t="inlineStr"/>
       <c r="L21" s="17" t="inlineStr"/>
+      <c r="M21" s="17" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L21"/>
+  <autoFilter ref="A1:M21"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId2"/>
@@ -7748,26 +7888,32 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId36"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7779,7 +7925,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:Q21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7798,6 +7944,7 @@
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7873,10 +8020,15 @@
       </c>
       <c r="O1" s="12" t="inlineStr">
         <is>
+          <t>prepared.gaps.output_path</t>
+        </is>
+      </c>
+      <c r="P1" s="12" t="inlineStr">
+        <is>
           <t>prepared.modeller.output_path</t>
         </is>
       </c>
-      <c r="P1" s="12" t="inlineStr">
+      <c r="Q1" s="12" t="inlineStr">
         <is>
           <t>prepared.alphafold.output_path</t>
         </is>
@@ -7947,6 +8099,7 @@
       </c>
       <c r="O2" s="13" t="inlineStr"/>
       <c r="P2" s="13" t="inlineStr"/>
+      <c r="Q2" s="13" t="inlineStr"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="16" t="inlineStr">
@@ -8013,6 +8166,7 @@
       </c>
       <c r="O3" s="17" t="inlineStr"/>
       <c r="P3" s="17" t="inlineStr"/>
+      <c r="Q3" s="17" t="inlineStr"/>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -8079,6 +8233,7 @@
       </c>
       <c r="O4" s="13" t="inlineStr"/>
       <c r="P4" s="13" t="inlineStr"/>
+      <c r="Q4" s="13" t="inlineStr"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="16" t="inlineStr">
@@ -8145,6 +8300,7 @@
       </c>
       <c r="O5" s="17" t="inlineStr"/>
       <c r="P5" s="17" t="inlineStr"/>
+      <c r="Q5" s="17" t="inlineStr"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -8218,7 +8374,8 @@
         </is>
       </c>
       <c r="O6" s="13" t="inlineStr"/>
-      <c r="P6" s="29" t="inlineStr">
+      <c r="P6" s="13" t="inlineStr"/>
+      <c r="Q6" s="29" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -8277,6 +8434,7 @@
       <c r="N7" s="17" t="inlineStr"/>
       <c r="O7" s="17" t="inlineStr"/>
       <c r="P7" s="17" t="inlineStr"/>
+      <c r="Q7" s="17" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="21" t="inlineStr">
@@ -8331,6 +8489,7 @@
       <c r="N8" s="13" t="inlineStr"/>
       <c r="O8" s="13" t="inlineStr"/>
       <c r="P8" s="13" t="inlineStr"/>
+      <c r="Q8" s="13" t="inlineStr"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="16" t="inlineStr">
@@ -8403,8 +8562,13 @@
           <t>open</t>
         </is>
       </c>
-      <c r="O9" s="17" t="inlineStr"/>
-      <c r="P9" s="30" t="inlineStr">
+      <c r="O9" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="P9" s="17" t="inlineStr"/>
+      <c r="Q9" s="30" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -8463,6 +8627,7 @@
       <c r="N10" s="13" t="inlineStr"/>
       <c r="O10" s="13" t="inlineStr"/>
       <c r="P10" s="13" t="inlineStr"/>
+      <c r="Q10" s="13" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="16" t="inlineStr">
@@ -8536,7 +8701,8 @@
         </is>
       </c>
       <c r="O11" s="17" t="inlineStr"/>
-      <c r="P11" s="30" t="inlineStr">
+      <c r="P11" s="17" t="inlineStr"/>
+      <c r="Q11" s="30" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -8618,7 +8784,12 @@
           <t>open</t>
         </is>
       </c>
-      <c r="P12" s="13" t="inlineStr"/>
+      <c r="P12" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Q12" s="13" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="19" t="inlineStr">
@@ -8673,6 +8844,7 @@
       <c r="N13" s="17" t="inlineStr"/>
       <c r="O13" s="17" t="inlineStr"/>
       <c r="P13" s="17" t="inlineStr"/>
+      <c r="Q13" s="17" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -8746,7 +8918,8 @@
         </is>
       </c>
       <c r="O14" s="13" t="inlineStr"/>
-      <c r="P14" s="29" t="inlineStr">
+      <c r="P14" s="13" t="inlineStr"/>
+      <c r="Q14" s="29" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -8805,9 +8978,10 @@
       <c r="N15" s="17" t="inlineStr"/>
       <c r="O15" s="17" t="inlineStr"/>
       <c r="P15" s="17" t="inlineStr"/>
+      <c r="Q15" s="17" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>3K5E</t>
         </is>
@@ -8833,7 +9007,11 @@
           <t>open</t>
         </is>
       </c>
-      <c r="G16" s="13" t="inlineStr"/>
+      <c r="G16" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="H16" s="13" t="inlineStr"/>
       <c r="I16" s="29" t="inlineStr">
         <is>
@@ -8855,10 +9033,23 @@
           <t>open</t>
         </is>
       </c>
-      <c r="M16" s="13" t="inlineStr"/>
-      <c r="N16" s="13" t="inlineStr"/>
-      <c r="O16" s="13" t="inlineStr"/>
+      <c r="M16" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="N16" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="O16" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="P16" s="13" t="inlineStr"/>
+      <c r="Q16" s="13" t="inlineStr"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
@@ -8925,6 +9116,7 @@
       </c>
       <c r="O17" s="17" t="inlineStr"/>
       <c r="P17" s="17" t="inlineStr"/>
+      <c r="Q17" s="17" t="inlineStr"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="21" t="inlineStr">
@@ -8979,6 +9171,7 @@
       <c r="N18" s="13" t="inlineStr"/>
       <c r="O18" s="13" t="inlineStr"/>
       <c r="P18" s="13" t="inlineStr"/>
+      <c r="Q18" s="13" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
@@ -9051,8 +9244,13 @@
           <t>open</t>
         </is>
       </c>
-      <c r="O19" s="17" t="inlineStr"/>
-      <c r="P19" s="30" t="inlineStr">
+      <c r="O19" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="P19" s="17" t="inlineStr"/>
+      <c r="Q19" s="30" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -9123,6 +9321,7 @@
       </c>
       <c r="O20" s="13" t="inlineStr"/>
       <c r="P20" s="13" t="inlineStr"/>
+      <c r="Q20" s="13" t="inlineStr"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="19" t="inlineStr">
@@ -9177,9 +9376,10 @@
       <c r="N21" s="17" t="inlineStr"/>
       <c r="O21" s="17" t="inlineStr"/>
       <c r="P21" s="17" t="inlineStr"/>
+      <c r="Q21" s="17" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P21"/>
+  <autoFilter ref="A1:Q21"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId2"/>
@@ -9238,7 +9438,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId61"/>
@@ -9268,133 +9468,140 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P9" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P11" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P14" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P19" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P12" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId221"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9406,7 +9613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY21"/>
+  <dimension ref="A1:BB21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9446,20 +9653,23 @@
     <col width="26" customWidth="1" min="35" max="35"/>
     <col width="12" customWidth="1" min="36" max="36"/>
     <col width="12" customWidth="1" min="37" max="37"/>
-    <col width="18" customWidth="1" min="38" max="38"/>
-    <col width="21" customWidth="1" min="39" max="39"/>
-    <col width="17" customWidth="1" min="40" max="40"/>
-    <col width="24" customWidth="1" min="41" max="41"/>
-    <col width="28" customWidth="1" min="42" max="42"/>
+    <col width="12" customWidth="1" min="38" max="38"/>
+    <col width="18" customWidth="1" min="39" max="39"/>
+    <col width="21" customWidth="1" min="40" max="40"/>
+    <col width="17" customWidth="1" min="41" max="41"/>
+    <col width="24" customWidth="1" min="42" max="42"/>
     <col width="28" customWidth="1" min="43" max="43"/>
     <col width="28" customWidth="1" min="44" max="44"/>
-    <col width="23" customWidth="1" min="45" max="45"/>
-    <col width="20" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="28" customWidth="1" min="45" max="45"/>
+    <col width="23" customWidth="1" min="46" max="46"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
     <col width="12" customWidth="1" min="48" max="48"/>
-    <col width="13" customWidth="1" min="49" max="49"/>
-    <col width="12" customWidth="1" min="50" max="50"/>
-    <col width="20" customWidth="1" min="51" max="51"/>
+    <col width="12" customWidth="1" min="49" max="49"/>
+    <col width="22" customWidth="1" min="50" max="50"/>
+    <col width="26" customWidth="1" min="51" max="51"/>
+    <col width="13" customWidth="1" min="52" max="52"/>
+    <col width="12" customWidth="1" min="53" max="53"/>
+    <col width="25" customWidth="1" min="54" max="54"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9640,80 +9850,95 @@
       </c>
       <c r="AJ1" s="12" t="inlineStr">
         <is>
+          <t>prepared.gaps.output_path</t>
+        </is>
+      </c>
+      <c r="AK1" s="12" t="inlineStr">
+        <is>
           <t>prepared.modeller.output_path</t>
         </is>
       </c>
-      <c r="AK1" s="12" t="inlineStr">
+      <c r="AL1" s="12" t="inlineStr">
         <is>
           <t>prepared.alphafold.output_path</t>
         </is>
       </c>
-      <c r="AL1" s="12" t="inlineStr">
+      <c r="AM1" s="12" t="inlineStr">
         <is>
           <t>available_models</t>
         </is>
       </c>
-      <c r="AM1" s="12" t="inlineStr">
+      <c r="AN1" s="12" t="inlineStr">
         <is>
           <t>metals_check.status</t>
         </is>
       </c>
-      <c r="AN1" s="12" t="inlineStr">
+      <c r="AO1" s="12" t="inlineStr">
         <is>
           <t>metals.ion_type</t>
         </is>
       </c>
-      <c r="AO1" s="12" t="inlineStr">
+      <c r="AP1" s="12" t="inlineStr">
         <is>
           <t>metals.class</t>
         </is>
       </c>
-      <c r="AP1" s="12" t="inlineStr">
+      <c r="AQ1" s="12" t="inlineStr">
         <is>
           <t>metals.parameter_reference</t>
         </is>
       </c>
-      <c r="AQ1" s="12" t="inlineStr">
+      <c r="AR1" s="12" t="inlineStr">
         <is>
           <t>metals.geometry_found</t>
         </is>
       </c>
-      <c r="AR1" s="12" t="inlineStr">
+      <c r="AS1" s="12" t="inlineStr">
         <is>
           <t>metals.geometry_probable</t>
         </is>
       </c>
-      <c r="AS1" s="12" t="inlineStr">
+      <c r="AT1" s="12" t="inlineStr">
         <is>
           <t>metals.geometry_match</t>
         </is>
       </c>
-      <c r="AT1" s="12" t="inlineStr">
+      <c r="AU1" s="12" t="inlineStr">
         <is>
           <t>metals.model_ready</t>
         </is>
       </c>
-      <c r="AU1" s="12" t="inlineStr">
+      <c r="AV1" s="12" t="inlineStr">
         <is>
           <t>metals.check_log_path</t>
         </is>
       </c>
-      <c r="AV1" s="12" t="inlineStr">
+      <c r="AW1" s="12" t="inlineStr">
         <is>
           <t>metals.check_manifest_path</t>
         </is>
       </c>
-      <c r="AW1" s="12" t="inlineStr">
+      <c r="AX1" s="12" t="inlineStr">
+        <is>
+          <t>metall_params.status</t>
+        </is>
+      </c>
+      <c r="AY1" s="12" t="inlineStr">
+        <is>
+          <t>metall_params.site_count</t>
+        </is>
+      </c>
+      <c r="AZ1" s="12" t="inlineStr">
         <is>
           <t>final_model</t>
         </is>
       </c>
-      <c r="AX1" s="12" t="inlineStr">
+      <c r="BA1" s="12" t="inlineStr">
         <is>
           <t>final_model_path</t>
         </is>
       </c>
-      <c r="AY1" s="12" t="inlineStr">
+      <c r="BB1" s="12" t="inlineStr">
         <is>
           <t>final_model_type</t>
         </is>
@@ -9885,19 +10110,15 @@
       </c>
       <c r="AJ2" s="13" t="inlineStr"/>
       <c r="AK2" s="13" t="inlineStr"/>
-      <c r="AL2" s="13" t="inlineStr">
+      <c r="AL2" s="13" t="inlineStr"/>
+      <c r="AM2" s="13" t="inlineStr">
         <is>
           <t>initial</t>
         </is>
       </c>
-      <c r="AM2" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="AN2" s="13" t="inlineStr">
-        <is>
-          <t>none</t>
+      <c r="AN2" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
         </is>
       </c>
       <c r="AO2" s="13" t="inlineStr">
@@ -9920,19 +10141,19 @@
           <t>none</t>
         </is>
       </c>
-      <c r="AS2" s="22" t="inlineStr">
+      <c r="AS2" s="13" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AT2" s="22" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="AT2" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AU2" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
+      <c r="AU2" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="AV2" s="29" t="inlineStr">
@@ -9940,17 +10161,24 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AW2" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AX2" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="AY2" s="13" t="inlineStr">
+      <c r="AW2" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AX2" s="13" t="inlineStr"/>
+      <c r="AY2" s="13" t="inlineStr"/>
+      <c r="AZ2" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA2" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BB2" s="13" t="inlineStr">
         <is>
           <t>single</t>
         </is>
@@ -10122,54 +10350,50 @@
       </c>
       <c r="AJ3" s="17" t="inlineStr"/>
       <c r="AK3" s="17" t="inlineStr"/>
-      <c r="AL3" s="17" t="inlineStr">
+      <c r="AL3" s="17" t="inlineStr"/>
+      <c r="AM3" s="17" t="inlineStr">
         <is>
           <t>initial</t>
         </is>
       </c>
-      <c r="AM3" s="15" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="AN3" s="17" t="inlineStr">
+      <c r="AN3" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AO3" s="17" t="inlineStr">
         <is>
           <t>Mg2+</t>
         </is>
       </c>
-      <c r="AO3" s="17" t="inlineStr">
+      <c r="AP3" s="17" t="inlineStr">
         <is>
           <t>standard_nontransition</t>
         </is>
       </c>
-      <c r="AP3" s="17" t="inlineStr">
+      <c r="AQ3" s="17" t="inlineStr">
         <is>
           <t>Standard AMBER divalent-ion route; not a Joung-Cheatham monovalent ion. Verify selected Mg2+ parameters against the water model.</t>
         </is>
       </c>
-      <c r="AQ3" s="17" t="inlineStr">
+      <c r="AR3" s="17" t="inlineStr">
         <is>
           <t>not_required_for_standard_ion</t>
         </is>
       </c>
-      <c r="AR3" s="17" t="inlineStr">
+      <c r="AS3" s="17" t="inlineStr">
         <is>
           <t>not_required_for_standard_ion</t>
         </is>
       </c>
-      <c r="AS3" s="23" t="inlineStr">
+      <c r="AT3" s="23" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="AT3" s="17" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AU3" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
+      <c r="AU3" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="AV3" s="30" t="inlineStr">
@@ -10177,17 +10401,32 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AW3" s="16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AX3" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="AY3" s="17" t="inlineStr">
+      <c r="AW3" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AX3" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="AY3" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AZ3" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA3" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BB3" s="17" t="inlineStr">
         <is>
           <t>single</t>
         </is>
@@ -10359,54 +10598,50 @@
       </c>
       <c r="AJ4" s="13" t="inlineStr"/>
       <c r="AK4" s="13" t="inlineStr"/>
-      <c r="AL4" s="13" t="inlineStr">
+      <c r="AL4" s="13" t="inlineStr"/>
+      <c r="AM4" s="13" t="inlineStr">
         <is>
           <t>initial</t>
         </is>
       </c>
-      <c r="AM4" s="15" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="AN4" s="13" t="inlineStr">
+      <c r="AN4" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AO4" s="13" t="inlineStr">
         <is>
           <t>Ca2+</t>
         </is>
       </c>
-      <c r="AO4" s="13" t="inlineStr">
+      <c r="AP4" s="13" t="inlineStr">
         <is>
           <t>standard_nontransition</t>
         </is>
       </c>
-      <c r="AP4" s="13" t="inlineStr">
+      <c r="AQ4" s="13" t="inlineStr">
         <is>
           <t>Standard AMBER divalent-ion route; not a Joung-Cheatham monovalent ion. Verify selected Ca2+ parameters against the water model.</t>
         </is>
       </c>
-      <c r="AQ4" s="13" t="inlineStr">
+      <c r="AR4" s="13" t="inlineStr">
         <is>
           <t>not_required_for_standard_ion</t>
         </is>
       </c>
-      <c r="AR4" s="13" t="inlineStr">
+      <c r="AS4" s="13" t="inlineStr">
         <is>
           <t>not_required_for_standard_ion</t>
         </is>
       </c>
-      <c r="AS4" s="22" t="inlineStr">
+      <c r="AT4" s="22" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="AT4" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AU4" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
+      <c r="AU4" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="AV4" s="29" t="inlineStr">
@@ -10414,17 +10649,32 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AW4" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AX4" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="AY4" s="13" t="inlineStr">
+      <c r="AW4" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AX4" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="AY4" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AZ4" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA4" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BB4" s="13" t="inlineStr">
         <is>
           <t>single</t>
         </is>
@@ -10596,19 +10846,15 @@
       </c>
       <c r="AJ5" s="17" t="inlineStr"/>
       <c r="AK5" s="17" t="inlineStr"/>
-      <c r="AL5" s="17" t="inlineStr">
+      <c r="AL5" s="17" t="inlineStr"/>
+      <c r="AM5" s="17" t="inlineStr">
         <is>
           <t>initial</t>
         </is>
       </c>
-      <c r="AM5" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="AN5" s="17" t="inlineStr">
-        <is>
-          <t>none</t>
+      <c r="AN5" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
         </is>
       </c>
       <c r="AO5" s="17" t="inlineStr">
@@ -10631,19 +10877,19 @@
           <t>none</t>
         </is>
       </c>
-      <c r="AS5" s="23" t="inlineStr">
+      <c r="AS5" s="17" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AT5" s="23" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="AT5" s="17" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AU5" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
+      <c r="AU5" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="AV5" s="30" t="inlineStr">
@@ -10651,17 +10897,24 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AW5" s="16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AX5" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="AY5" s="17" t="inlineStr">
+      <c r="AW5" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AX5" s="17" t="inlineStr"/>
+      <c r="AY5" s="17" t="inlineStr"/>
+      <c r="AZ5" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA5" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BB5" s="17" t="inlineStr">
         <is>
           <t>single</t>
         </is>
@@ -10844,24 +11097,20 @@
         </is>
       </c>
       <c r="AJ6" s="13" t="inlineStr"/>
-      <c r="AK6" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="AL6" s="13" t="inlineStr">
+      <c r="AK6" s="13" t="inlineStr"/>
+      <c r="AL6" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AM6" s="13" t="inlineStr">
         <is>
           <t>alphafold</t>
         </is>
       </c>
-      <c r="AM6" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="AN6" s="13" t="inlineStr">
-        <is>
-          <t>none</t>
+      <c r="AN6" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
         </is>
       </c>
       <c r="AO6" s="13" t="inlineStr">
@@ -10884,19 +11133,19 @@
           <t>none</t>
         </is>
       </c>
-      <c r="AS6" s="22" t="inlineStr">
+      <c r="AS6" s="13" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AT6" s="22" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="AT6" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AU6" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
+      <c r="AU6" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="AV6" s="29" t="inlineStr">
@@ -10904,17 +11153,24 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AW6" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AX6" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="AY6" s="13" t="inlineStr">
+      <c r="AW6" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AX6" s="13" t="inlineStr"/>
+      <c r="AY6" s="13" t="inlineStr"/>
+      <c r="AZ6" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA6" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BB6" s="13" t="inlineStr">
         <is>
           <t>best_complete</t>
         </is>
@@ -11075,49 +11331,45 @@
       <c r="AJ7" s="17" t="inlineStr"/>
       <c r="AK7" s="17" t="inlineStr"/>
       <c r="AL7" s="17" t="inlineStr"/>
-      <c r="AM7" s="18" t="inlineStr">
+      <c r="AM7" s="17" t="inlineStr"/>
+      <c r="AN7" s="18" t="inlineStr">
         <is>
           <t>required</t>
         </is>
       </c>
-      <c r="AN7" s="17" t="inlineStr">
+      <c r="AO7" s="17" t="inlineStr">
         <is>
           <t>Zn2+</t>
         </is>
       </c>
-      <c r="AO7" s="17" t="inlineStr">
+      <c r="AP7" s="17" t="inlineStr">
         <is>
           <t>transition</t>
         </is>
       </c>
-      <c r="AP7" s="17" t="inlineStr">
+      <c r="AQ7" s="17" t="inlineStr">
         <is>
           <t>transition-metal parameters required; geometry recorded for Gaussian/RESP/CESGA branch</t>
         </is>
       </c>
-      <c r="AQ7" s="24" t="inlineStr">
+      <c r="AR7" s="24" t="inlineStr">
         <is>
           <t>tetrahedral</t>
         </is>
       </c>
-      <c r="AR7" s="24" t="inlineStr">
+      <c r="AS7" s="24" t="inlineStr">
         <is>
           <t>tetrahedral|trigonal_bipyramidal|octahedral</t>
         </is>
       </c>
-      <c r="AS7" s="25" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AT7" s="17" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AU7" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
+      <c r="AT7" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AU7" s="17" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="AV7" s="30" t="inlineStr">
@@ -11125,13 +11377,28 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AW7" s="19" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AX7" s="17" t="inlineStr"/>
-      <c r="AY7" s="17" t="inlineStr"/>
+      <c r="AW7" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AX7" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="AY7" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AZ7" s="19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BA7" s="17" t="inlineStr"/>
+      <c r="BB7" s="17" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="21" t="inlineStr">
@@ -11288,49 +11555,45 @@
       <c r="AJ8" s="13" t="inlineStr"/>
       <c r="AK8" s="13" t="inlineStr"/>
       <c r="AL8" s="13" t="inlineStr"/>
-      <c r="AM8" s="18" t="inlineStr">
+      <c r="AM8" s="13" t="inlineStr"/>
+      <c r="AN8" s="18" t="inlineStr">
         <is>
           <t>required</t>
         </is>
       </c>
-      <c r="AN8" s="13" t="inlineStr">
+      <c r="AO8" s="13" t="inlineStr">
         <is>
           <t>Zn2+</t>
         </is>
       </c>
-      <c r="AO8" s="13" t="inlineStr">
+      <c r="AP8" s="13" t="inlineStr">
         <is>
           <t>transition</t>
         </is>
       </c>
-      <c r="AP8" s="13" t="inlineStr">
+      <c r="AQ8" s="13" t="inlineStr">
         <is>
           <t>transition-metal parameters required; geometry recorded for Gaussian/RESP/CESGA branch</t>
         </is>
       </c>
-      <c r="AQ8" s="26" t="inlineStr">
+      <c r="AR8" s="26" t="inlineStr">
         <is>
           <t>octahedral</t>
         </is>
       </c>
-      <c r="AR8" s="26" t="inlineStr">
+      <c r="AS8" s="26" t="inlineStr">
         <is>
           <t>tetrahedral|trigonal_bipyramidal|octahedral</t>
         </is>
       </c>
-      <c r="AS8" s="27" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AT8" s="13" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AU8" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
+      <c r="AT8" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AU8" s="13" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="AV8" s="29" t="inlineStr">
@@ -11338,13 +11601,28 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AW8" s="21" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AX8" s="13" t="inlineStr"/>
-      <c r="AY8" s="13" t="inlineStr"/>
+      <c r="AW8" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AX8" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="AY8" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AZ8" s="21" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BA8" s="13" t="inlineStr"/>
+      <c r="BB8" s="13" t="inlineStr"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="16" t="inlineStr">
@@ -11489,7 +11767,7 @@
       </c>
       <c r="AC9" s="17" t="inlineStr">
         <is>
-          <t>large_gap_complete</t>
+          <t>gaps,large_gap_complete</t>
         </is>
       </c>
       <c r="AD9" s="30" t="inlineStr">
@@ -11522,25 +11800,25 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="AJ9" s="17" t="inlineStr"/>
-      <c r="AK9" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="AL9" s="17" t="inlineStr">
-        <is>
-          <t>alphafold</t>
-        </is>
-      </c>
-      <c r="AM9" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="AN9" s="17" t="inlineStr">
-        <is>
-          <t>none</t>
+      <c r="AJ9" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AK9" s="17" t="inlineStr"/>
+      <c r="AL9" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AM9" s="17" t="inlineStr">
+        <is>
+          <t>gaps | alphafold</t>
+        </is>
+      </c>
+      <c r="AN9" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
         </is>
       </c>
       <c r="AO9" s="17" t="inlineStr">
@@ -11563,19 +11841,19 @@
           <t>none</t>
         </is>
       </c>
-      <c r="AS9" s="23" t="inlineStr">
+      <c r="AS9" s="17" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AT9" s="23" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="AT9" s="17" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AU9" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
+      <c r="AU9" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="AV9" s="30" t="inlineStr">
@@ -11583,19 +11861,26 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AW9" s="16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AX9" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="AY9" s="17" t="inlineStr">
-        <is>
-          <t>large_gap_complete</t>
+      <c r="AW9" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AX9" s="17" t="inlineStr"/>
+      <c r="AY9" s="17" t="inlineStr"/>
+      <c r="AZ9" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA9" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BB9" s="17" t="inlineStr">
+        <is>
+          <t>gaps,large_gap_complete</t>
         </is>
       </c>
     </row>
@@ -11754,14 +12039,10 @@
       <c r="AJ10" s="13" t="inlineStr"/>
       <c r="AK10" s="13" t="inlineStr"/>
       <c r="AL10" s="13" t="inlineStr"/>
-      <c r="AM10" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="AN10" s="13" t="inlineStr">
-        <is>
-          <t>none</t>
+      <c r="AM10" s="13" t="inlineStr"/>
+      <c r="AN10" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
         </is>
       </c>
       <c r="AO10" s="13" t="inlineStr">
@@ -11784,19 +12065,19 @@
           <t>none</t>
         </is>
       </c>
-      <c r="AS10" s="22" t="inlineStr">
+      <c r="AS10" s="13" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AT10" s="22" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="AT10" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AU10" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
+      <c r="AU10" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="AV10" s="29" t="inlineStr">
@@ -11804,13 +12085,20 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AW10" s="21" t="inlineStr">
-        <is>
-          <t>no</t>
+      <c r="AW10" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
         </is>
       </c>
       <c r="AX10" s="13" t="inlineStr"/>
       <c r="AY10" s="13" t="inlineStr"/>
+      <c r="AZ10" s="21" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BA10" s="13" t="inlineStr"/>
+      <c r="BB10" s="13" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="16" t="inlineStr">
@@ -11989,24 +12277,20 @@
         </is>
       </c>
       <c r="AJ11" s="17" t="inlineStr"/>
-      <c r="AK11" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="AL11" s="17" t="inlineStr">
+      <c r="AK11" s="17" t="inlineStr"/>
+      <c r="AL11" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AM11" s="17" t="inlineStr">
         <is>
           <t>alphafold</t>
         </is>
       </c>
-      <c r="AM11" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="AN11" s="17" t="inlineStr">
-        <is>
-          <t>none</t>
+      <c r="AN11" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
         </is>
       </c>
       <c r="AO11" s="17" t="inlineStr">
@@ -12029,19 +12313,19 @@
           <t>none</t>
         </is>
       </c>
-      <c r="AS11" s="23" t="inlineStr">
+      <c r="AS11" s="17" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AT11" s="23" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="AT11" s="17" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AU11" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
+      <c r="AU11" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="AV11" s="30" t="inlineStr">
@@ -12049,17 +12333,24 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AW11" s="16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AX11" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="AY11" s="17" t="inlineStr">
+      <c r="AW11" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AX11" s="17" t="inlineStr"/>
+      <c r="AY11" s="17" t="inlineStr"/>
+      <c r="AZ11" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA11" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BB11" s="17" t="inlineStr">
         <is>
           <t>best_complete</t>
         </is>
@@ -12208,7 +12499,7 @@
       </c>
       <c r="AC12" s="13" t="inlineStr">
         <is>
-          <t>best_complete</t>
+          <t>gaps,best_complete</t>
         </is>
       </c>
       <c r="AD12" s="29" t="inlineStr">
@@ -12246,20 +12537,20 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AK12" s="13" t="inlineStr"/>
-      <c r="AL12" s="13" t="inlineStr">
-        <is>
-          <t>modeller</t>
-        </is>
-      </c>
-      <c r="AM12" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="AN12" s="13" t="inlineStr">
-        <is>
-          <t>none</t>
+      <c r="AK12" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AL12" s="13" t="inlineStr"/>
+      <c r="AM12" s="13" t="inlineStr">
+        <is>
+          <t>gaps | modeller</t>
+        </is>
+      </c>
+      <c r="AN12" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
         </is>
       </c>
       <c r="AO12" s="13" t="inlineStr">
@@ -12282,19 +12573,19 @@
           <t>none</t>
         </is>
       </c>
-      <c r="AS12" s="22" t="inlineStr">
+      <c r="AS12" s="13" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AT12" s="22" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="AT12" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AU12" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
+      <c r="AU12" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="AV12" s="29" t="inlineStr">
@@ -12302,19 +12593,26 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AW12" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AX12" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="AY12" s="13" t="inlineStr">
-        <is>
-          <t>best_complete</t>
+      <c r="AW12" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AX12" s="13" t="inlineStr"/>
+      <c r="AY12" s="13" t="inlineStr"/>
+      <c r="AZ12" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA12" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BB12" s="13" t="inlineStr">
+        <is>
+          <t>gaps,best_complete</t>
         </is>
       </c>
     </row>
@@ -12473,49 +12771,45 @@
       <c r="AJ13" s="17" t="inlineStr"/>
       <c r="AK13" s="17" t="inlineStr"/>
       <c r="AL13" s="17" t="inlineStr"/>
-      <c r="AM13" s="18" t="inlineStr">
+      <c r="AM13" s="17" t="inlineStr"/>
+      <c r="AN13" s="18" t="inlineStr">
         <is>
           <t>required</t>
         </is>
       </c>
-      <c r="AN13" s="17" t="inlineStr">
+      <c r="AO13" s="17" t="inlineStr">
         <is>
           <t>Zn2+</t>
         </is>
       </c>
-      <c r="AO13" s="17" t="inlineStr">
+      <c r="AP13" s="17" t="inlineStr">
         <is>
           <t>transition</t>
         </is>
       </c>
-      <c r="AP13" s="17" t="inlineStr">
+      <c r="AQ13" s="17" t="inlineStr">
         <is>
           <t>transition-metal parameters required; geometry recorded for Gaussian/RESP/CESGA branch</t>
         </is>
       </c>
-      <c r="AQ13" s="28" t="inlineStr">
+      <c r="AR13" s="28" t="inlineStr">
         <is>
           <t>trigonal_planar</t>
         </is>
       </c>
-      <c r="AR13" s="28" t="inlineStr">
+      <c r="AS13" s="28" t="inlineStr">
         <is>
           <t>tetrahedral|trigonal_bipyramidal|octahedral</t>
         </is>
       </c>
-      <c r="AS13" s="19" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AT13" s="17" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AU13" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
+      <c r="AT13" s="19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU13" s="17" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="AV13" s="30" t="inlineStr">
@@ -12523,13 +12817,28 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AW13" s="19" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AX13" s="17" t="inlineStr"/>
-      <c r="AY13" s="17" t="inlineStr"/>
+      <c r="AW13" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AX13" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="AY13" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AZ13" s="19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BA13" s="17" t="inlineStr"/>
+      <c r="BB13" s="17" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -12708,24 +13017,20 @@
         </is>
       </c>
       <c r="AJ14" s="13" t="inlineStr"/>
-      <c r="AK14" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="AL14" s="13" t="inlineStr">
+      <c r="AK14" s="13" t="inlineStr"/>
+      <c r="AL14" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AM14" s="13" t="inlineStr">
         <is>
           <t>alphafold</t>
         </is>
       </c>
-      <c r="AM14" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="AN14" s="13" t="inlineStr">
-        <is>
-          <t>none</t>
+      <c r="AN14" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
         </is>
       </c>
       <c r="AO14" s="13" t="inlineStr">
@@ -12748,19 +13053,19 @@
           <t>none</t>
         </is>
       </c>
-      <c r="AS14" s="22" t="inlineStr">
+      <c r="AS14" s="13" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AT14" s="22" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="AT14" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AU14" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
+      <c r="AU14" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="AV14" s="29" t="inlineStr">
@@ -12768,17 +13073,24 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AW14" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AX14" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="AY14" s="13" t="inlineStr">
+      <c r="AW14" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AX14" s="13" t="inlineStr"/>
+      <c r="AY14" s="13" t="inlineStr"/>
+      <c r="AZ14" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA14" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BB14" s="13" t="inlineStr">
         <is>
           <t>best_complete</t>
         </is>
@@ -12939,49 +13251,45 @@
       <c r="AJ15" s="17" t="inlineStr"/>
       <c r="AK15" s="17" t="inlineStr"/>
       <c r="AL15" s="17" t="inlineStr"/>
-      <c r="AM15" s="18" t="inlineStr">
+      <c r="AM15" s="17" t="inlineStr"/>
+      <c r="AN15" s="18" t="inlineStr">
         <is>
           <t>required</t>
         </is>
       </c>
-      <c r="AN15" s="17" t="inlineStr">
+      <c r="AO15" s="17" t="inlineStr">
         <is>
           <t>Zn2+; Mg2+</t>
         </is>
       </c>
-      <c r="AO15" s="17" t="inlineStr">
+      <c r="AP15" s="17" t="inlineStr">
         <is>
           <t>mixed</t>
         </is>
       </c>
-      <c r="AP15" s="17" t="inlineStr">
+      <c r="AQ15" s="17" t="inlineStr">
         <is>
           <t>transition-metal parameters required; geometry recorded for Gaussian/RESP/CESGA branch; Standard AMBER divalent-ion route; not a Joung-Cheatham monovalent ion. Verify selected Mg2+ parameters against the water model.</t>
         </is>
       </c>
-      <c r="AQ15" s="24" t="inlineStr">
+      <c r="AR15" s="24" t="inlineStr">
         <is>
           <t>trigonal_bipyramidal; not_required_for_standard_ion</t>
         </is>
       </c>
-      <c r="AR15" s="24" t="inlineStr">
+      <c r="AS15" s="24" t="inlineStr">
         <is>
           <t>tetrahedral|trigonal_bipyramidal|octahedral; not_required_for_standard_ion</t>
         </is>
       </c>
-      <c r="AS15" s="25" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AT15" s="17" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AU15" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
+      <c r="AT15" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AU15" s="17" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="AV15" s="30" t="inlineStr">
@@ -12989,16 +13297,31 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AW15" s="19" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AX15" s="17" t="inlineStr"/>
-      <c r="AY15" s="17" t="inlineStr"/>
+      <c r="AW15" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AX15" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="AY15" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AZ15" s="19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BA15" s="17" t="inlineStr"/>
+      <c r="BB15" s="17" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>3K5E</t>
         </is>
@@ -13121,14 +13444,26 @@
           <t>skipped</t>
         </is>
       </c>
-      <c r="AB16" s="20" t="inlineStr">
-        <is>
-          <t>failed</t>
-        </is>
-      </c>
-      <c r="AC16" s="13" t="inlineStr"/>
-      <c r="AD16" s="13" t="inlineStr"/>
-      <c r="AE16" s="13" t="inlineStr"/>
+      <c r="AB16" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AC16" s="13" t="inlineStr">
+        <is>
+          <t>gaps</t>
+        </is>
+      </c>
+      <c r="AD16" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AE16" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AF16" s="13" t="inlineStr">
         <is>
           <t>gaps_only_no_complete_model</t>
@@ -13149,52 +13484,56 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AJ16" s="13" t="inlineStr"/>
+      <c r="AJ16" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AK16" s="13" t="inlineStr"/>
       <c r="AL16" s="13" t="inlineStr"/>
-      <c r="AM16" s="15" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="AN16" s="13" t="inlineStr">
+      <c r="AM16" s="13" t="inlineStr">
+        <is>
+          <t>gaps</t>
+        </is>
+      </c>
+      <c r="AN16" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AO16" s="13" t="inlineStr">
         <is>
           <t>Mg2+</t>
         </is>
       </c>
-      <c r="AO16" s="13" t="inlineStr">
+      <c r="AP16" s="13" t="inlineStr">
         <is>
           <t>standard_nontransition</t>
         </is>
       </c>
-      <c r="AP16" s="13" t="inlineStr">
+      <c r="AQ16" s="13" t="inlineStr">
         <is>
           <t>Standard AMBER divalent-ion route; not a Joung-Cheatham monovalent ion. Verify selected Mg2+ parameters against the water model.</t>
         </is>
       </c>
-      <c r="AQ16" s="13" t="inlineStr">
+      <c r="AR16" s="13" t="inlineStr">
         <is>
           <t>not_required_for_standard_ion</t>
         </is>
       </c>
-      <c r="AR16" s="13" t="inlineStr">
+      <c r="AS16" s="13" t="inlineStr">
         <is>
           <t>not_required_for_standard_ion</t>
         </is>
       </c>
-      <c r="AS16" s="22" t="inlineStr">
+      <c r="AT16" s="22" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="AT16" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AU16" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
+      <c r="AU16" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="AV16" s="29" t="inlineStr">
@@ -13202,13 +13541,36 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AW16" s="21" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AX16" s="13" t="inlineStr"/>
-      <c r="AY16" s="13" t="inlineStr"/>
+      <c r="AW16" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AX16" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="AY16" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AZ16" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA16" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BB16" s="13" t="inlineStr">
+        <is>
+          <t>gaps</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
@@ -13376,19 +13738,15 @@
       </c>
       <c r="AJ17" s="17" t="inlineStr"/>
       <c r="AK17" s="17" t="inlineStr"/>
-      <c r="AL17" s="17" t="inlineStr">
+      <c r="AL17" s="17" t="inlineStr"/>
+      <c r="AM17" s="17" t="inlineStr">
         <is>
           <t>initial</t>
         </is>
       </c>
-      <c r="AM17" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="AN17" s="17" t="inlineStr">
-        <is>
-          <t>none</t>
+      <c r="AN17" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
         </is>
       </c>
       <c r="AO17" s="17" t="inlineStr">
@@ -13411,19 +13769,19 @@
           <t>none</t>
         </is>
       </c>
-      <c r="AS17" s="23" t="inlineStr">
+      <c r="AS17" s="17" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AT17" s="23" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="AT17" s="17" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AU17" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
+      <c r="AU17" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="AV17" s="30" t="inlineStr">
@@ -13431,17 +13789,24 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AW17" s="16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AX17" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="AY17" s="17" t="inlineStr">
+      <c r="AW17" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AX17" s="17" t="inlineStr"/>
+      <c r="AY17" s="17" t="inlineStr"/>
+      <c r="AZ17" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA17" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BB17" s="17" t="inlineStr">
         <is>
           <t>single</t>
         </is>
@@ -13602,14 +13967,10 @@
       <c r="AJ18" s="13" t="inlineStr"/>
       <c r="AK18" s="13" t="inlineStr"/>
       <c r="AL18" s="13" t="inlineStr"/>
-      <c r="AM18" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="AN18" s="13" t="inlineStr">
-        <is>
-          <t>none</t>
+      <c r="AM18" s="13" t="inlineStr"/>
+      <c r="AN18" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
         </is>
       </c>
       <c r="AO18" s="13" t="inlineStr">
@@ -13632,19 +13993,19 @@
           <t>none</t>
         </is>
       </c>
-      <c r="AS18" s="22" t="inlineStr">
+      <c r="AS18" s="13" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AT18" s="22" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="AT18" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AU18" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
+      <c r="AU18" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="AV18" s="29" t="inlineStr">
@@ -13652,13 +14013,20 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AW18" s="21" t="inlineStr">
-        <is>
-          <t>no</t>
+      <c r="AW18" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
         </is>
       </c>
       <c r="AX18" s="13" t="inlineStr"/>
       <c r="AY18" s="13" t="inlineStr"/>
+      <c r="AZ18" s="21" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BA18" s="13" t="inlineStr"/>
+      <c r="BB18" s="13" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
@@ -13803,7 +14171,7 @@
       </c>
       <c r="AC19" s="17" t="inlineStr">
         <is>
-          <t>best_complete</t>
+          <t>gaps,best_complete</t>
         </is>
       </c>
       <c r="AD19" s="30" t="inlineStr">
@@ -13836,25 +14204,25 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="AJ19" s="17" t="inlineStr"/>
-      <c r="AK19" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="AL19" s="17" t="inlineStr">
-        <is>
-          <t>alphafold</t>
-        </is>
-      </c>
-      <c r="AM19" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="AN19" s="17" t="inlineStr">
-        <is>
-          <t>none</t>
+      <c r="AJ19" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AK19" s="17" t="inlineStr"/>
+      <c r="AL19" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AM19" s="17" t="inlineStr">
+        <is>
+          <t>gaps | alphafold</t>
+        </is>
+      </c>
+      <c r="AN19" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
         </is>
       </c>
       <c r="AO19" s="17" t="inlineStr">
@@ -13877,19 +14245,19 @@
           <t>none</t>
         </is>
       </c>
-      <c r="AS19" s="23" t="inlineStr">
+      <c r="AS19" s="17" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AT19" s="23" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="AT19" s="17" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AU19" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
+      <c r="AU19" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="AV19" s="30" t="inlineStr">
@@ -13897,19 +14265,26 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AW19" s="16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AX19" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="AY19" s="17" t="inlineStr">
-        <is>
-          <t>best_complete</t>
+      <c r="AW19" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AX19" s="17" t="inlineStr"/>
+      <c r="AY19" s="17" t="inlineStr"/>
+      <c r="AZ19" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA19" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BB19" s="17" t="inlineStr">
+        <is>
+          <t>gaps,best_complete</t>
         </is>
       </c>
     </row>
@@ -14079,19 +14454,15 @@
       </c>
       <c r="AJ20" s="13" t="inlineStr"/>
       <c r="AK20" s="13" t="inlineStr"/>
-      <c r="AL20" s="13" t="inlineStr">
+      <c r="AL20" s="13" t="inlineStr"/>
+      <c r="AM20" s="13" t="inlineStr">
         <is>
           <t>initial</t>
         </is>
       </c>
-      <c r="AM20" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="AN20" s="13" t="inlineStr">
-        <is>
-          <t>none</t>
+      <c r="AN20" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
         </is>
       </c>
       <c r="AO20" s="13" t="inlineStr">
@@ -14114,19 +14485,19 @@
           <t>none</t>
         </is>
       </c>
-      <c r="AS20" s="22" t="inlineStr">
+      <c r="AS20" s="13" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AT20" s="22" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="AT20" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AU20" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
+      <c r="AU20" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="AV20" s="29" t="inlineStr">
@@ -14134,17 +14505,24 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AW20" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AX20" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="AY20" s="13" t="inlineStr">
+      <c r="AW20" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AX20" s="13" t="inlineStr"/>
+      <c r="AY20" s="13" t="inlineStr"/>
+      <c r="AZ20" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA20" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BB20" s="13" t="inlineStr">
         <is>
           <t>single</t>
         </is>
@@ -14305,49 +14683,45 @@
       <c r="AJ21" s="17" t="inlineStr"/>
       <c r="AK21" s="17" t="inlineStr"/>
       <c r="AL21" s="17" t="inlineStr"/>
-      <c r="AM21" s="15" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="AN21" s="17" t="inlineStr">
+      <c r="AM21" s="17" t="inlineStr"/>
+      <c r="AN21" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="AO21" s="17" t="inlineStr">
         <is>
           <t>Na+; Na+</t>
         </is>
       </c>
-      <c r="AO21" s="17" t="inlineStr">
+      <c r="AP21" s="17" t="inlineStr">
         <is>
           <t>standard_nontransition</t>
         </is>
       </c>
-      <c r="AP21" s="17" t="inlineStr">
+      <c r="AQ21" s="17" t="inlineStr">
         <is>
           <t>Joung-Cheatham monovalent ion parameters; verify water-model-specific frcmod, e.g. ionsjc_tip3p for TIP3P.</t>
         </is>
       </c>
-      <c r="AQ21" s="17" t="inlineStr">
+      <c r="AR21" s="17" t="inlineStr">
         <is>
           <t>not_required_for_standard_ion; not_required_for_standard_ion</t>
         </is>
       </c>
-      <c r="AR21" s="17" t="inlineStr">
+      <c r="AS21" s="17" t="inlineStr">
         <is>
           <t>not_required_for_standard_ion; not_required_for_standard_ion</t>
         </is>
       </c>
-      <c r="AS21" s="23" t="inlineStr">
+      <c r="AT21" s="23" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="AT21" s="17" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AU21" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
+      <c r="AU21" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="AV21" s="30" t="inlineStr">
@@ -14355,16 +14729,31 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AW21" s="19" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AX21" s="17" t="inlineStr"/>
-      <c r="AY21" s="17" t="inlineStr"/>
+      <c r="AW21" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AX21" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="AY21" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AZ21" s="19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BA21" s="17" t="inlineStr"/>
+      <c r="BB21" s="17" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AY21"/>
+  <autoFilter ref="A1:BB21"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
@@ -14375,9 +14764,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z2" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD2" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE2" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AU2" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV2" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX2" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV2" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW2" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA2" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId15"/>
@@ -14387,219 +14776,234 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z3" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD3" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE3" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AU3" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV3" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX3" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y4" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z4" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD4" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE4" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AU4" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV3" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW3" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY3" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA3" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y4" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z4" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD4" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE4" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV4" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX4" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y5" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z5" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD5" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE5" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AU5" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV5" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX5" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U6" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y6" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z6" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD6" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE6" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK6" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AU6" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV6" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX6" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y7" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z7" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AU7" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV7" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y8" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z8" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AU8" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV8" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U9" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y9" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z9" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD9" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE9" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK9" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AU9" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV9" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX9" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y10" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z10" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AU10" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV10" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U11" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y11" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z11" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD11" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE11" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK11" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AU11" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV11" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX11" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U12" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y12" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z12" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD12" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE12" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ12" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AU12" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV12" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX12" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y13" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z13" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AU13" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV13" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U14" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y14" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z14" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD14" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE14" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK14" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AU14" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV14" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX14" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y15" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z15" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AU15" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV15" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y16" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z16" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AU16" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV16" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y17" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z17" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD17" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE17" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AU17" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV17" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX17" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y18" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z18" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AU18" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV18" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U19" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y19" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z19" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD19" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE19" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK19" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AU19" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV19" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX19" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y20" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z20" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD20" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE20" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AU20" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV20" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX20" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y21" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z21" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AU21" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV21" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW4" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY4" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA4" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y5" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z5" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD5" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE5" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV5" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW5" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA5" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U6" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y6" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z6" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD6" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE6" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL6" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV6" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW6" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA6" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y7" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z7" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV7" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW7" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY7" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y8" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z8" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV8" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW8" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY8" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U9" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y9" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z9" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD9" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE9" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ9" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL9" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV9" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW9" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA9" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y10" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z10" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV10" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW10" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U11" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y11" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z11" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD11" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE11" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL11" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV11" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW11" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA11" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U12" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y12" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z12" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD12" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE12" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ12" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK12" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV12" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW12" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA12" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y13" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z13" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV13" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW13" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY13" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U14" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y14" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z14" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD14" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE14" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL14" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV14" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW14" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA14" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y15" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z15" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV15" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW15" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY15" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y16" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z16" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD16" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE16" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ16" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV16" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW16" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY16" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA16" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y17" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z17" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD17" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE17" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV17" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW17" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA17" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y18" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z18" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV18" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW18" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U19" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y19" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z19" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD19" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE19" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ19" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL19" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV19" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW19" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA19" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y20" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z20" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD20" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE20" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV20" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW20" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA20" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y21" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z21" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV21" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW21" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY21" r:id="rId249"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: regenerate metall_params scaffolds after filename and input-selection fix
1W4R (ZN, tetrahedral) and 3FRG (ZN, tetrahedral) produce full MCPB
scaffolds with auto-filled ion_ids, ZN.mol2, and charge_m_sm = 2 1.
2AFX (ZN + ligand 1BN) and 3EWJ (ZN, non-standard geometry) correctly
write GEOMETRY_MISMATCH.txt and skip the MCPB scaffold.
1B8O (Mg), 1F0R (Ca), 3K5E (Mg), 3RM2 (Na) are correctly skipped as
non-transition metals that use standard force-field non-bonded params.
</commit_message>
<xml_diff>
--- a/data/proteins/pipeline.xlsx
+++ b/data/proteins/pipeline.xlsx
@@ -24,7 +24,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'chemistry'!$A$1:$M$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'prepared_outputs'!$A$1:$M$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'paths'!$A$1:$Q$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'full_state'!$A$1:$BB$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'full_state'!$A$1:$BC$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -5870,9 +5870,9 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="M7" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
         </is>
       </c>
     </row>
@@ -5937,9 +5937,9 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="M8" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
+      <c r="M8" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
         </is>
       </c>
     </row>
@@ -6256,9 +6256,9 @@
           <t>no</t>
         </is>
       </c>
-      <c r="M13" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
         </is>
       </c>
     </row>
@@ -6386,9 +6386,9 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="M15" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
         </is>
       </c>
     </row>
@@ -9613,7 +9613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB21"/>
+  <dimension ref="A1:BC21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9667,9 +9667,10 @@
     <col width="12" customWidth="1" min="49" max="49"/>
     <col width="22" customWidth="1" min="50" max="50"/>
     <col width="26" customWidth="1" min="51" max="51"/>
-    <col width="13" customWidth="1" min="52" max="52"/>
-    <col width="12" customWidth="1" min="53" max="53"/>
-    <col width="25" customWidth="1" min="54" max="54"/>
+    <col width="12" customWidth="1" min="52" max="52"/>
+    <col width="13" customWidth="1" min="53" max="53"/>
+    <col width="12" customWidth="1" min="54" max="54"/>
+    <col width="25" customWidth="1" min="55" max="55"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9930,15 +9931,20 @@
       </c>
       <c r="AZ1" s="12" t="inlineStr">
         <is>
+          <t>metall_params.manifest_path</t>
+        </is>
+      </c>
+      <c r="BA1" s="12" t="inlineStr">
+        <is>
           <t>final_model</t>
         </is>
       </c>
-      <c r="BA1" s="12" t="inlineStr">
+      <c r="BB1" s="12" t="inlineStr">
         <is>
           <t>final_model_path</t>
         </is>
       </c>
-      <c r="BB1" s="12" t="inlineStr">
+      <c r="BC1" s="12" t="inlineStr">
         <is>
           <t>final_model_type</t>
         </is>
@@ -10168,17 +10174,18 @@
       </c>
       <c r="AX2" s="13" t="inlineStr"/>
       <c r="AY2" s="13" t="inlineStr"/>
-      <c r="AZ2" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BA2" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BB2" s="13" t="inlineStr">
+      <c r="AZ2" s="13" t="inlineStr"/>
+      <c r="BA2" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB2" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BC2" s="13" t="inlineStr">
         <is>
           <t>single</t>
         </is>
@@ -10416,17 +10423,18 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AZ3" s="16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BA3" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BB3" s="17" t="inlineStr">
+      <c r="AZ3" s="17" t="inlineStr"/>
+      <c r="BA3" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB3" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BC3" s="17" t="inlineStr">
         <is>
           <t>single</t>
         </is>
@@ -10664,17 +10672,18 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AZ4" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BA4" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BB4" s="13" t="inlineStr">
+      <c r="AZ4" s="13" t="inlineStr"/>
+      <c r="BA4" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB4" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BC4" s="13" t="inlineStr">
         <is>
           <t>single</t>
         </is>
@@ -10904,17 +10913,18 @@
       </c>
       <c r="AX5" s="17" t="inlineStr"/>
       <c r="AY5" s="17" t="inlineStr"/>
-      <c r="AZ5" s="16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BA5" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BB5" s="17" t="inlineStr">
+      <c r="AZ5" s="17" t="inlineStr"/>
+      <c r="BA5" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB5" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BC5" s="17" t="inlineStr">
         <is>
           <t>single</t>
         </is>
@@ -11160,17 +11170,18 @@
       </c>
       <c r="AX6" s="13" t="inlineStr"/>
       <c r="AY6" s="13" t="inlineStr"/>
-      <c r="AZ6" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BA6" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BB6" s="13" t="inlineStr">
+      <c r="AZ6" s="13" t="inlineStr"/>
+      <c r="BA6" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB6" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BC6" s="13" t="inlineStr">
         <is>
           <t>best_complete</t>
         </is>
@@ -11382,9 +11393,9 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AX7" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
+      <c r="AX7" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
         </is>
       </c>
       <c r="AY7" s="30" t="inlineStr">
@@ -11392,13 +11403,18 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AZ7" s="19" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="BA7" s="17" t="inlineStr"/>
+      <c r="AZ7" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BA7" s="19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="BB7" s="17" t="inlineStr"/>
+      <c r="BC7" s="17" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="21" t="inlineStr">
@@ -11606,9 +11622,9 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AX8" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
+      <c r="AX8" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
         </is>
       </c>
       <c r="AY8" s="29" t="inlineStr">
@@ -11616,13 +11632,18 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AZ8" s="21" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="BA8" s="13" t="inlineStr"/>
+      <c r="AZ8" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BA8" s="21" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="BB8" s="13" t="inlineStr"/>
+      <c r="BC8" s="13" t="inlineStr"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="16" t="inlineStr">
@@ -11868,17 +11889,18 @@
       </c>
       <c r="AX9" s="17" t="inlineStr"/>
       <c r="AY9" s="17" t="inlineStr"/>
-      <c r="AZ9" s="16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BA9" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BB9" s="17" t="inlineStr">
+      <c r="AZ9" s="17" t="inlineStr"/>
+      <c r="BA9" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB9" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BC9" s="17" t="inlineStr">
         <is>
           <t>gaps,large_gap_complete</t>
         </is>
@@ -12092,13 +12114,14 @@
       </c>
       <c r="AX10" s="13" t="inlineStr"/>
       <c r="AY10" s="13" t="inlineStr"/>
-      <c r="AZ10" s="21" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="BA10" s="13" t="inlineStr"/>
+      <c r="AZ10" s="13" t="inlineStr"/>
+      <c r="BA10" s="21" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="BB10" s="13" t="inlineStr"/>
+      <c r="BC10" s="13" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="16" t="inlineStr">
@@ -12340,17 +12363,18 @@
       </c>
       <c r="AX11" s="17" t="inlineStr"/>
       <c r="AY11" s="17" t="inlineStr"/>
-      <c r="AZ11" s="16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BA11" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BB11" s="17" t="inlineStr">
+      <c r="AZ11" s="17" t="inlineStr"/>
+      <c r="BA11" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB11" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BC11" s="17" t="inlineStr">
         <is>
           <t>best_complete</t>
         </is>
@@ -12600,17 +12624,18 @@
       </c>
       <c r="AX12" s="13" t="inlineStr"/>
       <c r="AY12" s="13" t="inlineStr"/>
-      <c r="AZ12" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BA12" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BB12" s="13" t="inlineStr">
+      <c r="AZ12" s="13" t="inlineStr"/>
+      <c r="BA12" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB12" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BC12" s="13" t="inlineStr">
         <is>
           <t>gaps,best_complete</t>
         </is>
@@ -12822,9 +12847,9 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AX13" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
+      <c r="AX13" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
         </is>
       </c>
       <c r="AY13" s="30" t="inlineStr">
@@ -12832,13 +12857,18 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AZ13" s="19" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="BA13" s="17" t="inlineStr"/>
+      <c r="AZ13" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BA13" s="19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="BB13" s="17" t="inlineStr"/>
+      <c r="BC13" s="17" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -13080,17 +13110,18 @@
       </c>
       <c r="AX14" s="13" t="inlineStr"/>
       <c r="AY14" s="13" t="inlineStr"/>
-      <c r="AZ14" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BA14" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BB14" s="13" t="inlineStr">
+      <c r="AZ14" s="13" t="inlineStr"/>
+      <c r="BA14" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB14" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BC14" s="13" t="inlineStr">
         <is>
           <t>best_complete</t>
         </is>
@@ -13302,9 +13333,9 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AX15" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
+      <c r="AX15" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
         </is>
       </c>
       <c r="AY15" s="30" t="inlineStr">
@@ -13312,13 +13343,18 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AZ15" s="19" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="BA15" s="17" t="inlineStr"/>
+      <c r="AZ15" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BA15" s="19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="BB15" s="17" t="inlineStr"/>
+      <c r="BC15" s="17" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -13556,17 +13592,18 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AZ16" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BA16" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BB16" s="13" t="inlineStr">
+      <c r="AZ16" s="13" t="inlineStr"/>
+      <c r="BA16" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB16" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BC16" s="13" t="inlineStr">
         <is>
           <t>gaps</t>
         </is>
@@ -13796,17 +13833,18 @@
       </c>
       <c r="AX17" s="17" t="inlineStr"/>
       <c r="AY17" s="17" t="inlineStr"/>
-      <c r="AZ17" s="16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BA17" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BB17" s="17" t="inlineStr">
+      <c r="AZ17" s="17" t="inlineStr"/>
+      <c r="BA17" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB17" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BC17" s="17" t="inlineStr">
         <is>
           <t>single</t>
         </is>
@@ -14020,13 +14058,14 @@
       </c>
       <c r="AX18" s="13" t="inlineStr"/>
       <c r="AY18" s="13" t="inlineStr"/>
-      <c r="AZ18" s="21" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="BA18" s="13" t="inlineStr"/>
+      <c r="AZ18" s="13" t="inlineStr"/>
+      <c r="BA18" s="21" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="BB18" s="13" t="inlineStr"/>
+      <c r="BC18" s="13" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
@@ -14272,17 +14311,18 @@
       </c>
       <c r="AX19" s="17" t="inlineStr"/>
       <c r="AY19" s="17" t="inlineStr"/>
-      <c r="AZ19" s="16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BA19" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BB19" s="17" t="inlineStr">
+      <c r="AZ19" s="17" t="inlineStr"/>
+      <c r="BA19" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB19" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BC19" s="17" t="inlineStr">
         <is>
           <t>gaps,best_complete</t>
         </is>
@@ -14512,17 +14552,18 @@
       </c>
       <c r="AX20" s="13" t="inlineStr"/>
       <c r="AY20" s="13" t="inlineStr"/>
-      <c r="AZ20" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BA20" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BB20" s="13" t="inlineStr">
+      <c r="AZ20" s="13" t="inlineStr"/>
+      <c r="BA20" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BB20" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BC20" s="13" t="inlineStr">
         <is>
           <t>single</t>
         </is>
@@ -14744,16 +14785,17 @@
           <t>open</t>
         </is>
       </c>
-      <c r="AZ21" s="19" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="BA21" s="17" t="inlineStr"/>
+      <c r="AZ21" s="17" t="inlineStr"/>
+      <c r="BA21" s="19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="BB21" s="17" t="inlineStr"/>
+      <c r="BC21" s="17" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BB21"/>
+  <autoFilter ref="A1:BC21"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
@@ -14766,7 +14808,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE2" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV2" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW2" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA2" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB2" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId15"/>
@@ -14779,7 +14821,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV3" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW3" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY3" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA3" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB3" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId28"/>
@@ -14792,7 +14834,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV4" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW4" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY4" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA4" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB4" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId41"/>
@@ -14804,7 +14846,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE5" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV5" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW5" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA5" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB5" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId53"/>
@@ -14819,7 +14861,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL6" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV6" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW6" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA6" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB6" r:id="rId65"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId68"/>
@@ -14830,180 +14872,184 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV7" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW7" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY7" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y8" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z8" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV8" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW8" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY8" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U9" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y9" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z9" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD9" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE9" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ9" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL9" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV9" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW9" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA9" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y10" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z10" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV10" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW10" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U11" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y11" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z11" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD11" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE11" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL11" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV11" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW11" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA11" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U12" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y12" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z12" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD12" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE12" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ12" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK12" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV12" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW12" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA12" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y13" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z13" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV13" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW13" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY13" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U14" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y14" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z14" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD14" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE14" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL14" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV14" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW14" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA14" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y15" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z15" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV15" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW15" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY15" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y16" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z16" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD16" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE16" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ16" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV16" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW16" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY16" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA16" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y17" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z17" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD17" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE17" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV17" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW17" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA17" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y18" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z18" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV18" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW18" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U19" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y19" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z19" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD19" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE19" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ19" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL19" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV19" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW19" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA19" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y20" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z20" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD20" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE20" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV20" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW20" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BA20" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y21" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z21" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV21" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW21" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY21" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ7" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y8" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z8" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV8" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW8" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY8" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ8" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U9" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y9" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z9" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD9" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE9" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ9" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL9" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV9" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW9" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB9" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y10" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z10" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV10" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW10" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U11" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y11" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z11" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD11" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE11" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL11" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV11" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW11" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB11" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U12" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y12" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z12" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD12" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE12" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ12" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK12" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV12" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW12" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB12" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y13" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z13" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV13" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW13" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY13" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ13" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U14" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y14" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z14" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD14" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE14" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL14" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV14" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW14" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB14" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y15" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z15" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV15" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW15" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY15" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ15" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y16" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z16" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD16" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE16" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ16" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV16" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW16" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY16" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB16" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y17" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z17" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD17" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE17" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV17" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW17" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB17" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y18" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z18" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV18" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW18" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U19" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y19" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z19" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD19" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE19" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ19" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL19" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV19" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW19" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB19" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y20" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z20" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD20" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE20" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV20" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW20" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB20" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y21" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z21" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV21" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW21" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY21" r:id="rId253"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: regenerate pipeline.json and pipeline.xlsx with nonstd_residue_params columns
overview sheet now shows metall_params.status and nonstd_residue_params.{status,n_residues}
beside the has_metals / has_nonstandard_residues flags.
3OLL and 3BC3 both show nonstd_residue_params.status=success, n_residues=1.
</commit_message>
<xml_diff>
--- a/data/proteins/pipeline.xlsx
+++ b/data/proteins/pipeline.xlsx
@@ -17,14 +17,14 @@
     <sheet name="full_state" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'overview'!$A$6:$O$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'overview'!$A$6:$R$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'preparation'!$A$1:$G$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'components'!$A$1:$I$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'components'!$A$1:$K$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'gaps_and_variants'!$A$1:$L$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'chemistry'!$A$1:$M$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'chemistry'!$A$1:$O$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'prepared_outputs'!$A$1:$M$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'paths'!$A$1:$Q$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'full_state'!$A$1:$BC$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'paths'!$A$1:$R$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'full_state'!$A$1:$BF$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -747,7 +747,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O26"/>
+  <dimension ref="A1:R26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -757,14 +757,17 @@
     <col width="25" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="15" customWidth="1" min="13" max="13"/>
-    <col width="27" customWidth="1" min="14" max="14"/>
-    <col width="28" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="27" customWidth="1" min="17" max="17"/>
+    <col width="28" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="31" customHeight="1">
@@ -786,7 +789,10 @@
       <c r="L1" s="3" t="n"/>
       <c r="M1" s="3" t="n"/>
       <c r="N1" s="3" t="n"/>
-      <c r="O1" s="4" t="n"/>
+      <c r="O1" s="3" t="n"/>
+      <c r="P1" s="3" t="n"/>
+      <c r="Q1" s="3" t="n"/>
+      <c r="R1" s="4" t="n"/>
     </row>
     <row r="2" ht="20.25" customHeight="1">
       <c r="A2" s="5" t="n"/>
@@ -807,7 +813,10 @@
       <c r="L2" s="3" t="n"/>
       <c r="M2" s="3" t="n"/>
       <c r="N2" s="3" t="n"/>
-      <c r="O2" s="4" t="n"/>
+      <c r="O2" s="3" t="n"/>
+      <c r="P2" s="3" t="n"/>
+      <c r="Q2" s="3" t="n"/>
+      <c r="R2" s="4" t="n"/>
     </row>
     <row r="3" ht="10.1" customHeight="1">
       <c r="A3" s="7" t="inlineStr"/>
@@ -870,6 +879,9 @@
         <v>9</v>
       </c>
       <c r="O4" s="11" t="n"/>
+      <c r="P4" s="11" t="n"/>
+      <c r="Q4" s="11" t="n"/>
+      <c r="R4" s="11" t="n"/>
     </row>
     <row r="5"/>
     <row r="6">
@@ -910,40 +922,55 @@
       </c>
       <c r="H6" s="12" t="inlineStr">
         <is>
+          <t>metall_params.status</t>
+        </is>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
           <t>has_nonstandard_residues</t>
         </is>
       </c>
-      <c r="I6" s="12" t="inlineStr">
+      <c r="J6" s="12" t="inlineStr">
+        <is>
+          <t>nonstd_residue_params.status</t>
+        </is>
+      </c>
+      <c r="K6" s="12" t="inlineStr">
+        <is>
+          <t>nonstd_residue_params.n_residues</t>
+        </is>
+      </c>
+      <c r="L6" s="12" t="inlineStr">
         <is>
           <t>has_ligands</t>
         </is>
       </c>
-      <c r="J6" s="12" t="inlineStr">
+      <c r="M6" s="12" t="inlineStr">
         <is>
           <t>has_gaps</t>
         </is>
       </c>
-      <c r="K6" s="12" t="inlineStr">
+      <c r="N6" s="12" t="inlineStr">
         <is>
           <t>n_gaps</t>
         </is>
       </c>
-      <c r="L6" s="12" t="inlineStr">
+      <c r="O6" s="12" t="inlineStr">
         <is>
           <t>gap_sizes</t>
         </is>
       </c>
-      <c r="M6" s="12" t="inlineStr">
+      <c r="P6" s="12" t="inlineStr">
         <is>
           <t>filler.status</t>
         </is>
       </c>
-      <c r="N6" s="12" t="inlineStr">
+      <c r="Q6" s="12" t="inlineStr">
         <is>
           <t>prepared_structure.status</t>
         </is>
       </c>
-      <c r="O6" s="12" t="inlineStr">
+      <c r="R6" s="12" t="inlineStr">
         <is>
           <t>prepared_structure.variant</t>
         </is>
@@ -985,42 +1012,45 @@
           <t>no</t>
         </is>
       </c>
-      <c r="H7" s="13" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="H7" s="13" t="inlineStr"/>
       <c r="I7" s="13" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J7" s="13" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K7" s="13" t="inlineStr">
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J7" s="13" t="inlineStr"/>
+      <c r="K7" s="13" t="inlineStr"/>
+      <c r="L7" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M7" s="13" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N7" s="13" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L7" s="13" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="M7" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="N7" s="15" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
       <c r="O7" s="13" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P7" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="Q7" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R7" s="13" t="inlineStr">
         <is>
           <t>single</t>
         </is>
@@ -1062,42 +1092,49 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H8" s="17" t="inlineStr">
-        <is>
-          <t>no</t>
+      <c r="H8" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
         </is>
       </c>
       <c r="I8" s="17" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J8" s="17" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K8" s="17" t="inlineStr">
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J8" s="17" t="inlineStr"/>
+      <c r="K8" s="17" t="inlineStr"/>
+      <c r="L8" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L8" s="17" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="M8" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="N8" s="15" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
       <c r="O8" s="17" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P8" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="Q8" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R8" s="17" t="inlineStr">
         <is>
           <t>single</t>
         </is>
@@ -1139,42 +1176,49 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H9" s="13" t="inlineStr">
-        <is>
-          <t>no</t>
+      <c r="H9" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
         </is>
       </c>
       <c r="I9" s="13" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J9" s="13" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K9" s="13" t="inlineStr">
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J9" s="13" t="inlineStr"/>
+      <c r="K9" s="13" t="inlineStr"/>
+      <c r="L9" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M9" s="13" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N9" s="13" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L9" s="13" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="M9" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="N9" s="15" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
       <c r="O9" s="13" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P9" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="Q9" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R9" s="13" t="inlineStr">
         <is>
           <t>single</t>
         </is>
@@ -1216,42 +1260,45 @@
           <t>no</t>
         </is>
       </c>
-      <c r="H10" s="17" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="H10" s="17" t="inlineStr"/>
       <c r="I10" s="17" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J10" s="17" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K10" s="17" t="inlineStr">
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J10" s="17" t="inlineStr"/>
+      <c r="K10" s="17" t="inlineStr"/>
+      <c r="L10" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L10" s="17" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="M10" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="N10" s="15" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
       <c r="O10" s="17" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P10" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="Q10" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R10" s="17" t="inlineStr">
         <is>
           <t>single</t>
         </is>
@@ -1293,42 +1340,45 @@
           <t>no</t>
         </is>
       </c>
-      <c r="H11" s="13" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="H11" s="13" t="inlineStr"/>
       <c r="I11" s="13" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J11" s="18" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="K11" s="18" t="inlineStr">
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J11" s="13" t="inlineStr"/>
+      <c r="K11" s="13" t="inlineStr"/>
+      <c r="L11" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M11" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N11" s="18" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="L11" s="18" t="inlineStr">
+      <c r="O11" s="18" t="inlineStr">
         <is>
           <t>2|8</t>
         </is>
       </c>
-      <c r="M11" s="15" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="N11" s="15" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="O11" s="13" t="inlineStr">
+      <c r="P11" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="Q11" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R11" s="13" t="inlineStr">
         <is>
           <t>best_complete</t>
         </is>
@@ -1362,42 +1412,49 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H12" s="17" t="inlineStr">
-        <is>
-          <t>no</t>
+      <c r="H12" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
         </is>
       </c>
       <c r="I12" s="17" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J12" s="17" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K12" s="17" t="inlineStr">
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J12" s="17" t="inlineStr"/>
+      <c r="K12" s="17" t="inlineStr"/>
+      <c r="L12" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L12" s="17" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="M12" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="N12" s="20" t="inlineStr">
+      <c r="O12" s="17" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P12" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="Q12" s="20" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
       </c>
-      <c r="O12" s="17" t="inlineStr"/>
+      <c r="R12" s="17" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="21" t="inlineStr">
@@ -1427,42 +1484,49 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H13" s="13" t="inlineStr">
-        <is>
-          <t>no</t>
+      <c r="H13" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
         </is>
       </c>
       <c r="I13" s="13" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J13" s="18" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="K13" s="18" t="inlineStr">
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J13" s="13" t="inlineStr"/>
+      <c r="K13" s="13" t="inlineStr"/>
+      <c r="L13" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M13" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N13" s="18" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="L13" s="18" t="inlineStr">
+      <c r="O13" s="18" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="M13" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="N13" s="20" t="inlineStr">
+      <c r="P13" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="Q13" s="20" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
       </c>
-      <c r="O13" s="13" t="inlineStr"/>
+      <c r="R13" s="13" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="16" t="inlineStr">
@@ -1500,42 +1564,45 @@
           <t>no</t>
         </is>
       </c>
-      <c r="H14" s="17" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="H14" s="17" t="inlineStr"/>
       <c r="I14" s="17" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J14" s="18" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="K14" s="18" t="inlineStr">
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J14" s="17" t="inlineStr"/>
+      <c r="K14" s="17" t="inlineStr"/>
+      <c r="L14" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N14" s="18" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="L14" s="18" t="inlineStr">
+      <c r="O14" s="18" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="M14" s="15" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="N14" s="15" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="O14" s="17" t="inlineStr">
+      <c r="P14" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="Q14" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R14" s="17" t="inlineStr">
         <is>
           <t>gaps,large_gap_complete</t>
         </is>
@@ -1569,42 +1636,45 @@
           <t>no</t>
         </is>
       </c>
-      <c r="H15" s="13" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="H15" s="13" t="inlineStr"/>
       <c r="I15" s="13" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J15" s="13" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K15" s="13" t="inlineStr">
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J15" s="13" t="inlineStr"/>
+      <c r="K15" s="13" t="inlineStr"/>
+      <c r="L15" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M15" s="13" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N15" s="13" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L15" s="13" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="M15" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="N15" s="20" t="inlineStr">
+      <c r="O15" s="13" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P15" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="Q15" s="20" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
       </c>
-      <c r="O15" s="13" t="inlineStr"/>
+      <c r="R15" s="13" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
@@ -1642,42 +1712,45 @@
           <t>no</t>
         </is>
       </c>
-      <c r="H16" s="17" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="H16" s="17" t="inlineStr"/>
       <c r="I16" s="17" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J16" s="18" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="K16" s="18" t="inlineStr">
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J16" s="17" t="inlineStr"/>
+      <c r="K16" s="17" t="inlineStr"/>
+      <c r="L16" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M16" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N16" s="18" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="L16" s="18" t="inlineStr">
+      <c r="O16" s="18" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="M16" s="15" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="N16" s="15" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="O16" s="17" t="inlineStr">
+      <c r="P16" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="Q16" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R16" s="17" t="inlineStr">
         <is>
           <t>best_complete</t>
         </is>
@@ -1719,42 +1792,53 @@
           <t>no</t>
         </is>
       </c>
-      <c r="H17" s="18" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I17" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J17" s="18" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="K17" s="18" t="inlineStr">
+      <c r="H17" s="13" t="inlineStr"/>
+      <c r="I17" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J17" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K17" s="13" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="L17" s="18" t="inlineStr">
+      <c r="L17" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M17" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N17" s="18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O17" s="18" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="M17" s="15" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="N17" s="15" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="O17" s="13" t="inlineStr">
+      <c r="P17" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="Q17" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R17" s="13" t="inlineStr">
         <is>
           <t>gaps,best_complete</t>
         </is>
@@ -1788,42 +1872,49 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H18" s="17" t="inlineStr">
-        <is>
-          <t>no</t>
+      <c r="H18" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
         </is>
       </c>
       <c r="I18" s="17" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J18" s="17" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K18" s="17" t="inlineStr">
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J18" s="17" t="inlineStr"/>
+      <c r="K18" s="17" t="inlineStr"/>
+      <c r="L18" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L18" s="17" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="M18" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="N18" s="20" t="inlineStr">
+      <c r="O18" s="17" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P18" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="Q18" s="20" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
       </c>
-      <c r="O18" s="17" t="inlineStr"/>
+      <c r="R18" s="17" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
@@ -1861,42 +1952,45 @@
           <t>no</t>
         </is>
       </c>
-      <c r="H19" s="13" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="H19" s="13" t="inlineStr"/>
       <c r="I19" s="13" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J19" s="18" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="K19" s="18" t="inlineStr">
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J19" s="13" t="inlineStr"/>
+      <c r="K19" s="13" t="inlineStr"/>
+      <c r="L19" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M19" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N19" s="18" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="L19" s="18" t="inlineStr">
+      <c r="O19" s="18" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="M19" s="15" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="N19" s="15" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="O19" s="13" t="inlineStr">
+      <c r="P19" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="Q19" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R19" s="13" t="inlineStr">
         <is>
           <t>best_complete</t>
         </is>
@@ -1930,42 +2024,49 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H20" s="17" t="inlineStr">
-        <is>
-          <t>no</t>
+      <c r="H20" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
         </is>
       </c>
       <c r="I20" s="17" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J20" s="17" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K20" s="17" t="inlineStr">
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J20" s="17" t="inlineStr"/>
+      <c r="K20" s="17" t="inlineStr"/>
+      <c r="L20" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L20" s="17" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="M20" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="N20" s="20" t="inlineStr">
+      <c r="O20" s="17" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P20" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="Q20" s="20" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
       </c>
-      <c r="O20" s="17" t="inlineStr"/>
+      <c r="R20" s="17" t="inlineStr"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
@@ -2003,42 +2104,49 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H21" s="13" t="inlineStr">
-        <is>
-          <t>no</t>
+      <c r="H21" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
         </is>
       </c>
       <c r="I21" s="13" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J21" s="18" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="K21" s="18" t="inlineStr">
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J21" s="13" t="inlineStr"/>
+      <c r="K21" s="13" t="inlineStr"/>
+      <c r="L21" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M21" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N21" s="18" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="L21" s="18" t="inlineStr">
+      <c r="O21" s="18" t="inlineStr">
         <is>
           <t>2|15</t>
         </is>
       </c>
-      <c r="M21" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="N21" s="15" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="O21" s="13" t="inlineStr">
+      <c r="P21" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="Q21" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R21" s="13" t="inlineStr">
         <is>
           <t>gaps</t>
         </is>
@@ -2080,42 +2188,45 @@
           <t>no</t>
         </is>
       </c>
-      <c r="H22" s="17" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="H22" s="17" t="inlineStr"/>
       <c r="I22" s="17" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J22" s="17" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K22" s="17" t="inlineStr">
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J22" s="17" t="inlineStr"/>
+      <c r="K22" s="17" t="inlineStr"/>
+      <c r="L22" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M22" s="17" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N22" s="17" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L22" s="17" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="M22" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="N22" s="15" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
       <c r="O22" s="17" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P22" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="Q22" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R22" s="17" t="inlineStr">
         <is>
           <t>single</t>
         </is>
@@ -2149,42 +2260,45 @@
           <t>no</t>
         </is>
       </c>
-      <c r="H23" s="13" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="H23" s="13" t="inlineStr"/>
       <c r="I23" s="13" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J23" s="13" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K23" s="13" t="inlineStr">
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J23" s="13" t="inlineStr"/>
+      <c r="K23" s="13" t="inlineStr"/>
+      <c r="L23" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M23" s="13" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N23" s="13" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L23" s="13" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="M23" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="N23" s="20" t="inlineStr">
+      <c r="O23" s="13" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P23" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="Q23" s="20" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
       </c>
-      <c r="O23" s="13" t="inlineStr"/>
+      <c r="R23" s="13" t="inlineStr"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="16" t="inlineStr">
@@ -2222,42 +2336,53 @@
           <t>no</t>
         </is>
       </c>
-      <c r="H24" s="18" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I24" s="17" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J24" s="18" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="K24" s="18" t="inlineStr">
+      <c r="H24" s="17" t="inlineStr"/>
+      <c r="I24" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J24" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K24" s="17" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="L24" s="18" t="inlineStr">
+      <c r="L24" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M24" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N24" s="18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O24" s="18" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="M24" s="15" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="N24" s="15" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="O24" s="17" t="inlineStr">
+      <c r="P24" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="Q24" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R24" s="17" t="inlineStr">
         <is>
           <t>gaps,best_complete</t>
         </is>
@@ -2299,42 +2424,45 @@
           <t>no</t>
         </is>
       </c>
-      <c r="H25" s="13" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="H25" s="13" t="inlineStr"/>
       <c r="I25" s="13" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J25" s="13" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K25" s="13" t="inlineStr">
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J25" s="13" t="inlineStr"/>
+      <c r="K25" s="13" t="inlineStr"/>
+      <c r="L25" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M25" s="13" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N25" s="13" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L25" s="13" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="M25" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="N25" s="15" t="inlineStr">
-        <is>
-          <t>success</t>
-        </is>
-      </c>
       <c r="O25" s="13" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P25" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="Q25" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="R25" s="13" t="inlineStr">
         <is>
           <t>single</t>
         </is>
@@ -2368,49 +2496,56 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H26" s="17" t="inlineStr">
-        <is>
-          <t>no</t>
+      <c r="H26" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
         </is>
       </c>
       <c r="I26" s="17" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J26" s="18" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="K26" s="18" t="inlineStr">
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J26" s="17" t="inlineStr"/>
+      <c r="K26" s="17" t="inlineStr"/>
+      <c r="L26" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M26" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N26" s="18" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="L26" s="18" t="inlineStr">
+      <c r="O26" s="18" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="M26" s="14" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="N26" s="20" t="inlineStr">
+      <c r="P26" s="14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="Q26" s="20" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
       </c>
-      <c r="O26" s="17" t="inlineStr"/>
+      <c r="R26" s="17" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A6:O26"/>
+  <autoFilter ref="A6:R26"/>
   <mergeCells count="4">
-    <mergeCell ref="B1:O1"/>
-    <mergeCell ref="B2:O2"/>
-    <mergeCell ref="A3:O3"/>
+    <mergeCell ref="B1:R1"/>
+    <mergeCell ref="B2:R2"/>
+    <mergeCell ref="A3:R3"/>
     <mergeCell ref="A1:A2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3169,7 +3304,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3181,6 +3316,8 @@
     <col width="28" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3229,6 +3366,16 @@
           <t>has_nonstandard_residues</t>
         </is>
       </c>
+      <c r="J1" s="12" t="inlineStr">
+        <is>
+          <t>nonstd_residue_params.status</t>
+        </is>
+      </c>
+      <c r="K1" s="12" t="inlineStr">
+        <is>
+          <t>nonstd_residue_params.n_residues</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="8" t="inlineStr">
@@ -3276,6 +3423,8 @@
           <t>no</t>
         </is>
       </c>
+      <c r="J2" s="13" t="inlineStr"/>
+      <c r="K2" s="13" t="inlineStr"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="16" t="inlineStr">
@@ -3323,6 +3472,8 @@
           <t>no</t>
         </is>
       </c>
+      <c r="J3" s="17" t="inlineStr"/>
+      <c r="K3" s="17" t="inlineStr"/>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -3370,6 +3521,8 @@
           <t>no</t>
         </is>
       </c>
+      <c r="J4" s="13" t="inlineStr"/>
+      <c r="K4" s="13" t="inlineStr"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="16" t="inlineStr">
@@ -3417,6 +3570,8 @@
           <t>no</t>
         </is>
       </c>
+      <c r="J5" s="17" t="inlineStr"/>
+      <c r="K5" s="17" t="inlineStr"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -3464,6 +3619,8 @@
           <t>no</t>
         </is>
       </c>
+      <c r="J6" s="13" t="inlineStr"/>
+      <c r="K6" s="13" t="inlineStr"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="19" t="inlineStr">
@@ -3511,6 +3668,8 @@
           <t>no</t>
         </is>
       </c>
+      <c r="J7" s="17" t="inlineStr"/>
+      <c r="K7" s="17" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="21" t="inlineStr">
@@ -3558,6 +3717,8 @@
           <t>no</t>
         </is>
       </c>
+      <c r="J8" s="13" t="inlineStr"/>
+      <c r="K8" s="13" t="inlineStr"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="16" t="inlineStr">
@@ -3605,6 +3766,8 @@
           <t>no</t>
         </is>
       </c>
+      <c r="J9" s="17" t="inlineStr"/>
+      <c r="K9" s="17" t="inlineStr"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="21" t="inlineStr">
@@ -3652,6 +3815,8 @@
           <t>no</t>
         </is>
       </c>
+      <c r="J10" s="13" t="inlineStr"/>
+      <c r="K10" s="13" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="16" t="inlineStr">
@@ -3699,6 +3864,8 @@
           <t>no</t>
         </is>
       </c>
+      <c r="J11" s="17" t="inlineStr"/>
+      <c r="K11" s="17" t="inlineStr"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -3746,6 +3913,16 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="J12" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K12" s="13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="19" t="inlineStr">
@@ -3793,6 +3970,8 @@
           <t>no</t>
         </is>
       </c>
+      <c r="J13" s="17" t="inlineStr"/>
+      <c r="K13" s="17" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -3840,6 +4019,8 @@
           <t>no</t>
         </is>
       </c>
+      <c r="J14" s="13" t="inlineStr"/>
+      <c r="K14" s="13" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="19" t="inlineStr">
@@ -3887,6 +4068,8 @@
           <t>no</t>
         </is>
       </c>
+      <c r="J15" s="17" t="inlineStr"/>
+      <c r="K15" s="17" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -3934,6 +4117,8 @@
           <t>no</t>
         </is>
       </c>
+      <c r="J16" s="13" t="inlineStr"/>
+      <c r="K16" s="13" t="inlineStr"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
@@ -3981,6 +4166,8 @@
           <t>no</t>
         </is>
       </c>
+      <c r="J17" s="17" t="inlineStr"/>
+      <c r="K17" s="17" t="inlineStr"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="21" t="inlineStr">
@@ -4028,6 +4215,8 @@
           <t>no</t>
         </is>
       </c>
+      <c r="J18" s="13" t="inlineStr"/>
+      <c r="K18" s="13" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
@@ -4075,6 +4264,16 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="J19" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K19" s="17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -4122,6 +4321,8 @@
           <t>no</t>
         </is>
       </c>
+      <c r="J20" s="13" t="inlineStr"/>
+      <c r="K20" s="13" t="inlineStr"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="19" t="inlineStr">
@@ -4169,9 +4370,11 @@
           <t>no</t>
         </is>
       </c>
+      <c r="J21" s="17" t="inlineStr"/>
+      <c r="K21" s="17" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I21"/>
+  <autoFilter ref="A1:K21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5401,7 +5604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5417,6 +5620,8 @@
     <col width="28" customWidth="1" min="11" max="11"/>
     <col width="23" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="28" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5485,6 +5690,16 @@
           <t>metall_params.status</t>
         </is>
       </c>
+      <c r="N1" s="12" t="inlineStr">
+        <is>
+          <t>nonstd_residue_params.status</t>
+        </is>
+      </c>
+      <c r="O1" s="12" t="inlineStr">
+        <is>
+          <t>nonstd_residue_params.n_residues</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="8" t="inlineStr">
@@ -5548,6 +5763,8 @@
         </is>
       </c>
       <c r="M2" s="13" t="inlineStr"/>
+      <c r="N2" s="13" t="inlineStr"/>
+      <c r="O2" s="13" t="inlineStr"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="16" t="inlineStr">
@@ -5615,6 +5832,8 @@
           <t>skipped</t>
         </is>
       </c>
+      <c r="N3" s="17" t="inlineStr"/>
+      <c r="O3" s="17" t="inlineStr"/>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -5682,6 +5901,8 @@
           <t>skipped</t>
         </is>
       </c>
+      <c r="N4" s="13" t="inlineStr"/>
+      <c r="O4" s="13" t="inlineStr"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="16" t="inlineStr">
@@ -5745,6 +5966,8 @@
         </is>
       </c>
       <c r="M5" s="17" t="inlineStr"/>
+      <c r="N5" s="17" t="inlineStr"/>
+      <c r="O5" s="17" t="inlineStr"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -5808,6 +6031,8 @@
         </is>
       </c>
       <c r="M6" s="13" t="inlineStr"/>
+      <c r="N6" s="13" t="inlineStr"/>
+      <c r="O6" s="13" t="inlineStr"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="19" t="inlineStr">
@@ -5875,6 +6100,8 @@
           <t>success</t>
         </is>
       </c>
+      <c r="N7" s="17" t="inlineStr"/>
+      <c r="O7" s="17" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="21" t="inlineStr">
@@ -5942,6 +6169,8 @@
           <t>success</t>
         </is>
       </c>
+      <c r="N8" s="13" t="inlineStr"/>
+      <c r="O8" s="13" t="inlineStr"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="16" t="inlineStr">
@@ -6005,6 +6234,8 @@
         </is>
       </c>
       <c r="M9" s="17" t="inlineStr"/>
+      <c r="N9" s="17" t="inlineStr"/>
+      <c r="O9" s="17" t="inlineStr"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="21" t="inlineStr">
@@ -6068,6 +6299,8 @@
         </is>
       </c>
       <c r="M10" s="13" t="inlineStr"/>
+      <c r="N10" s="13" t="inlineStr"/>
+      <c r="O10" s="13" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="16" t="inlineStr">
@@ -6131,6 +6364,8 @@
         </is>
       </c>
       <c r="M11" s="17" t="inlineStr"/>
+      <c r="N11" s="17" t="inlineStr"/>
+      <c r="O11" s="17" t="inlineStr"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -6194,6 +6429,16 @@
         </is>
       </c>
       <c r="M12" s="13" t="inlineStr"/>
+      <c r="N12" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="O12" s="13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="19" t="inlineStr">
@@ -6261,6 +6506,8 @@
           <t>success</t>
         </is>
       </c>
+      <c r="N13" s="17" t="inlineStr"/>
+      <c r="O13" s="17" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -6324,6 +6571,8 @@
         </is>
       </c>
       <c r="M14" s="13" t="inlineStr"/>
+      <c r="N14" s="13" t="inlineStr"/>
+      <c r="O14" s="13" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="19" t="inlineStr">
@@ -6391,6 +6640,8 @@
           <t>success</t>
         </is>
       </c>
+      <c r="N15" s="17" t="inlineStr"/>
+      <c r="O15" s="17" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -6458,6 +6709,8 @@
           <t>skipped</t>
         </is>
       </c>
+      <c r="N16" s="13" t="inlineStr"/>
+      <c r="O16" s="13" t="inlineStr"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
@@ -6521,6 +6774,8 @@
         </is>
       </c>
       <c r="M17" s="17" t="inlineStr"/>
+      <c r="N17" s="17" t="inlineStr"/>
+      <c r="O17" s="17" t="inlineStr"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="21" t="inlineStr">
@@ -6584,6 +6839,8 @@
         </is>
       </c>
       <c r="M18" s="13" t="inlineStr"/>
+      <c r="N18" s="13" t="inlineStr"/>
+      <c r="O18" s="13" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
@@ -6647,6 +6904,16 @@
         </is>
       </c>
       <c r="M19" s="17" t="inlineStr"/>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="O19" s="17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -6710,6 +6977,8 @@
         </is>
       </c>
       <c r="M20" s="13" t="inlineStr"/>
+      <c r="N20" s="13" t="inlineStr"/>
+      <c r="O20" s="13" t="inlineStr"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="19" t="inlineStr">
@@ -6777,9 +7046,11 @@
           <t>skipped</t>
         </is>
       </c>
+      <c r="N21" s="17" t="inlineStr"/>
+      <c r="O21" s="17" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M21"/>
+  <autoFilter ref="A1:O21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7925,7 +8196,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q21"/>
+  <dimension ref="A1:R21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7945,6 +8216,7 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8000,35 +8272,40 @@
       </c>
       <c r="K1" s="12" t="inlineStr">
         <is>
+          <t>nonstd_residue_params.manifest_path</t>
+        </is>
+      </c>
+      <c r="L1" s="12" t="inlineStr">
+        <is>
           <t>protonation.input_path</t>
         </is>
       </c>
-      <c r="L1" s="12" t="inlineStr">
+      <c r="M1" s="12" t="inlineStr">
         <is>
           <t>protonation.output_path</t>
         </is>
       </c>
-      <c r="M1" s="12" t="inlineStr">
+      <c r="N1" s="12" t="inlineStr">
         <is>
           <t>prepared_structure.protein_input_path</t>
         </is>
       </c>
-      <c r="N1" s="12" t="inlineStr">
+      <c r="O1" s="12" t="inlineStr">
         <is>
           <t>prepared_structure.output_path</t>
         </is>
       </c>
-      <c r="O1" s="12" t="inlineStr">
+      <c r="P1" s="12" t="inlineStr">
         <is>
           <t>prepared.gaps.output_path</t>
         </is>
       </c>
-      <c r="P1" s="12" t="inlineStr">
+      <c r="Q1" s="12" t="inlineStr">
         <is>
           <t>prepared.modeller.output_path</t>
         </is>
       </c>
-      <c r="Q1" s="12" t="inlineStr">
+      <c r="R1" s="12" t="inlineStr">
         <is>
           <t>prepared.alphafold.output_path</t>
         </is>
@@ -8077,11 +8354,7 @@
           <t>open</t>
         </is>
       </c>
-      <c r="K2" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
+      <c r="K2" s="13" t="inlineStr"/>
       <c r="L2" s="29" t="inlineStr">
         <is>
           <t>open</t>
@@ -8097,9 +8370,14 @@
           <t>open</t>
         </is>
       </c>
-      <c r="O2" s="13" t="inlineStr"/>
+      <c r="O2" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="P2" s="13" t="inlineStr"/>
       <c r="Q2" s="13" t="inlineStr"/>
+      <c r="R2" s="13" t="inlineStr"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="16" t="inlineStr">
@@ -8144,11 +8422,7 @@
           <t>open</t>
         </is>
       </c>
-      <c r="K3" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
+      <c r="K3" s="17" t="inlineStr"/>
       <c r="L3" s="30" t="inlineStr">
         <is>
           <t>open</t>
@@ -8164,9 +8438,14 @@
           <t>open</t>
         </is>
       </c>
-      <c r="O3" s="17" t="inlineStr"/>
+      <c r="O3" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="P3" s="17" t="inlineStr"/>
       <c r="Q3" s="17" t="inlineStr"/>
+      <c r="R3" s="17" t="inlineStr"/>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -8211,11 +8490,7 @@
           <t>open</t>
         </is>
       </c>
-      <c r="K4" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
+      <c r="K4" s="13" t="inlineStr"/>
       <c r="L4" s="29" t="inlineStr">
         <is>
           <t>open</t>
@@ -8231,9 +8506,14 @@
           <t>open</t>
         </is>
       </c>
-      <c r="O4" s="13" t="inlineStr"/>
+      <c r="O4" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="P4" s="13" t="inlineStr"/>
       <c r="Q4" s="13" t="inlineStr"/>
+      <c r="R4" s="13" t="inlineStr"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="16" t="inlineStr">
@@ -8278,11 +8558,7 @@
           <t>open</t>
         </is>
       </c>
-      <c r="K5" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
+      <c r="K5" s="17" t="inlineStr"/>
       <c r="L5" s="30" t="inlineStr">
         <is>
           <t>open</t>
@@ -8298,9 +8574,14 @@
           <t>open</t>
         </is>
       </c>
-      <c r="O5" s="17" t="inlineStr"/>
+      <c r="O5" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="P5" s="17" t="inlineStr"/>
       <c r="Q5" s="17" t="inlineStr"/>
+      <c r="R5" s="17" t="inlineStr"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -8353,11 +8634,7 @@
           <t>open</t>
         </is>
       </c>
-      <c r="K6" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
+      <c r="K6" s="13" t="inlineStr"/>
       <c r="L6" s="29" t="inlineStr">
         <is>
           <t>open</t>
@@ -8373,9 +8650,14 @@
           <t>open</t>
         </is>
       </c>
-      <c r="O6" s="13" t="inlineStr"/>
+      <c r="O6" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="P6" s="13" t="inlineStr"/>
-      <c r="Q6" s="29" t="inlineStr">
+      <c r="Q6" s="13" t="inlineStr"/>
+      <c r="R6" s="29" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -8420,21 +8702,22 @@
           <t>open</t>
         </is>
       </c>
-      <c r="K7" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
+      <c r="K7" s="17" t="inlineStr"/>
       <c r="L7" s="30" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="M7" s="17" t="inlineStr"/>
+      <c r="M7" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="N7" s="17" t="inlineStr"/>
       <c r="O7" s="17" t="inlineStr"/>
       <c r="P7" s="17" t="inlineStr"/>
       <c r="Q7" s="17" t="inlineStr"/>
+      <c r="R7" s="17" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="21" t="inlineStr">
@@ -8475,21 +8758,22 @@
           <t>open</t>
         </is>
       </c>
-      <c r="K8" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
+      <c r="K8" s="13" t="inlineStr"/>
       <c r="L8" s="29" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="M8" s="13" t="inlineStr"/>
+      <c r="M8" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="N8" s="13" t="inlineStr"/>
       <c r="O8" s="13" t="inlineStr"/>
       <c r="P8" s="13" t="inlineStr"/>
       <c r="Q8" s="13" t="inlineStr"/>
+      <c r="R8" s="13" t="inlineStr"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="16" t="inlineStr">
@@ -8542,11 +8826,7 @@
           <t>open</t>
         </is>
       </c>
-      <c r="K9" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
+      <c r="K9" s="17" t="inlineStr"/>
       <c r="L9" s="30" t="inlineStr">
         <is>
           <t>open</t>
@@ -8567,8 +8847,13 @@
           <t>open</t>
         </is>
       </c>
-      <c r="P9" s="17" t="inlineStr"/>
-      <c r="Q9" s="30" t="inlineStr">
+      <c r="P9" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Q9" s="17" t="inlineStr"/>
+      <c r="R9" s="30" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -8613,21 +8898,22 @@
           <t>open</t>
         </is>
       </c>
-      <c r="K10" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
+      <c r="K10" s="13" t="inlineStr"/>
       <c r="L10" s="29" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="M10" s="13" t="inlineStr"/>
+      <c r="M10" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="N10" s="13" t="inlineStr"/>
       <c r="O10" s="13" t="inlineStr"/>
       <c r="P10" s="13" t="inlineStr"/>
       <c r="Q10" s="13" t="inlineStr"/>
+      <c r="R10" s="13" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="16" t="inlineStr">
@@ -8680,11 +8966,7 @@
           <t>open</t>
         </is>
       </c>
-      <c r="K11" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
+      <c r="K11" s="17" t="inlineStr"/>
       <c r="L11" s="30" t="inlineStr">
         <is>
           <t>open</t>
@@ -8700,9 +8982,14 @@
           <t>open</t>
         </is>
       </c>
-      <c r="O11" s="17" t="inlineStr"/>
+      <c r="O11" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="P11" s="17" t="inlineStr"/>
-      <c r="Q11" s="30" t="inlineStr">
+      <c r="Q11" s="17" t="inlineStr"/>
+      <c r="R11" s="30" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -8789,7 +9076,12 @@
           <t>open</t>
         </is>
       </c>
-      <c r="Q12" s="13" t="inlineStr"/>
+      <c r="Q12" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="R12" s="13" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="19" t="inlineStr">
@@ -8830,21 +9122,22 @@
           <t>open</t>
         </is>
       </c>
-      <c r="K13" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
+      <c r="K13" s="17" t="inlineStr"/>
       <c r="L13" s="30" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="M13" s="17" t="inlineStr"/>
+      <c r="M13" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="N13" s="17" t="inlineStr"/>
       <c r="O13" s="17" t="inlineStr"/>
       <c r="P13" s="17" t="inlineStr"/>
       <c r="Q13" s="17" t="inlineStr"/>
+      <c r="R13" s="17" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -8897,11 +9190,7 @@
           <t>open</t>
         </is>
       </c>
-      <c r="K14" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
+      <c r="K14" s="13" t="inlineStr"/>
       <c r="L14" s="29" t="inlineStr">
         <is>
           <t>open</t>
@@ -8917,9 +9206,14 @@
           <t>open</t>
         </is>
       </c>
-      <c r="O14" s="13" t="inlineStr"/>
+      <c r="O14" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="P14" s="13" t="inlineStr"/>
-      <c r="Q14" s="29" t="inlineStr">
+      <c r="Q14" s="13" t="inlineStr"/>
+      <c r="R14" s="29" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -8964,21 +9258,22 @@
           <t>open</t>
         </is>
       </c>
-      <c r="K15" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
+      <c r="K15" s="17" t="inlineStr"/>
       <c r="L15" s="30" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="M15" s="17" t="inlineStr"/>
+      <c r="M15" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="N15" s="17" t="inlineStr"/>
       <c r="O15" s="17" t="inlineStr"/>
       <c r="P15" s="17" t="inlineStr"/>
       <c r="Q15" s="17" t="inlineStr"/>
+      <c r="R15" s="17" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -9023,11 +9318,7 @@
           <t>open</t>
         </is>
       </c>
-      <c r="K16" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
+      <c r="K16" s="13" t="inlineStr"/>
       <c r="L16" s="29" t="inlineStr">
         <is>
           <t>open</t>
@@ -9048,8 +9339,13 @@
           <t>open</t>
         </is>
       </c>
-      <c r="P16" s="13" t="inlineStr"/>
+      <c r="P16" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Q16" s="13" t="inlineStr"/>
+      <c r="R16" s="13" t="inlineStr"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
@@ -9094,11 +9390,7 @@
           <t>open</t>
         </is>
       </c>
-      <c r="K17" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
+      <c r="K17" s="17" t="inlineStr"/>
       <c r="L17" s="30" t="inlineStr">
         <is>
           <t>open</t>
@@ -9114,9 +9406,14 @@
           <t>open</t>
         </is>
       </c>
-      <c r="O17" s="17" t="inlineStr"/>
+      <c r="O17" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="P17" s="17" t="inlineStr"/>
       <c r="Q17" s="17" t="inlineStr"/>
+      <c r="R17" s="17" t="inlineStr"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="21" t="inlineStr">
@@ -9157,21 +9454,22 @@
           <t>open</t>
         </is>
       </c>
-      <c r="K18" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
+      <c r="K18" s="13" t="inlineStr"/>
       <c r="L18" s="29" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="M18" s="13" t="inlineStr"/>
+      <c r="M18" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="N18" s="13" t="inlineStr"/>
       <c r="O18" s="13" t="inlineStr"/>
       <c r="P18" s="13" t="inlineStr"/>
       <c r="Q18" s="13" t="inlineStr"/>
+      <c r="R18" s="13" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
@@ -9249,8 +9547,13 @@
           <t>open</t>
         </is>
       </c>
-      <c r="P19" s="17" t="inlineStr"/>
-      <c r="Q19" s="30" t="inlineStr">
+      <c r="P19" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Q19" s="17" t="inlineStr"/>
+      <c r="R19" s="30" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -9299,11 +9602,7 @@
           <t>open</t>
         </is>
       </c>
-      <c r="K20" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
+      <c r="K20" s="13" t="inlineStr"/>
       <c r="L20" s="29" t="inlineStr">
         <is>
           <t>open</t>
@@ -9319,9 +9618,14 @@
           <t>open</t>
         </is>
       </c>
-      <c r="O20" s="13" t="inlineStr"/>
+      <c r="O20" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="P20" s="13" t="inlineStr"/>
       <c r="Q20" s="13" t="inlineStr"/>
+      <c r="R20" s="13" t="inlineStr"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="19" t="inlineStr">
@@ -9362,24 +9666,25 @@
           <t>open</t>
         </is>
       </c>
-      <c r="K21" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
+      <c r="K21" s="17" t="inlineStr"/>
       <c r="L21" s="30" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="M21" s="17" t="inlineStr"/>
+      <c r="M21" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="N21" s="17" t="inlineStr"/>
       <c r="O21" s="17" t="inlineStr"/>
       <c r="P21" s="17" t="inlineStr"/>
       <c r="Q21" s="17" t="inlineStr"/>
+      <c r="R21" s="17" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q21"/>
+  <autoFilter ref="A1:R21"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId2"/>
@@ -9388,10 +9693,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId14"/>
@@ -9399,10 +9704,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId25"/>
@@ -9410,10 +9715,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId36"/>
@@ -9421,10 +9726,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId47"/>
@@ -9434,27 +9739,27 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId69"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId70"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId75"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId77"/>
@@ -9464,20 +9769,20 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId81"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId82"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P9" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId89"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId90"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId91"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId92"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId93"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId94"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId97"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId98"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId99"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId100"/>
@@ -9487,11 +9792,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId104"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId105"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId111"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId112"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId113"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId114"/>
@@ -9507,101 +9812,103 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId124"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId125"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P12" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId133"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId144"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId145"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId146"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId155"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId164"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId165"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId166"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId167"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P16" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId176"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId177"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId178"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId186"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P19" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId223"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9613,7 +9920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BC21"/>
+  <dimension ref="A1:BF21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9668,9 +9975,12 @@
     <col width="22" customWidth="1" min="50" max="50"/>
     <col width="26" customWidth="1" min="51" max="51"/>
     <col width="12" customWidth="1" min="52" max="52"/>
-    <col width="13" customWidth="1" min="53" max="53"/>
-    <col width="12" customWidth="1" min="54" max="54"/>
-    <col width="25" customWidth="1" min="55" max="55"/>
+    <col width="28" customWidth="1" min="53" max="53"/>
+    <col width="28" customWidth="1" min="54" max="54"/>
+    <col width="12" customWidth="1" min="55" max="55"/>
+    <col width="13" customWidth="1" min="56" max="56"/>
+    <col width="12" customWidth="1" min="57" max="57"/>
+    <col width="25" customWidth="1" min="58" max="58"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9936,15 +10246,30 @@
       </c>
       <c r="BA1" s="12" t="inlineStr">
         <is>
+          <t>nonstd_residue_params.status</t>
+        </is>
+      </c>
+      <c r="BB1" s="12" t="inlineStr">
+        <is>
+          <t>nonstd_residue_params.n_residues</t>
+        </is>
+      </c>
+      <c r="BC1" s="12" t="inlineStr">
+        <is>
+          <t>nonstd_residue_params.manifest_path</t>
+        </is>
+      </c>
+      <c r="BD1" s="12" t="inlineStr">
+        <is>
           <t>final_model</t>
         </is>
       </c>
-      <c r="BB1" s="12" t="inlineStr">
+      <c r="BE1" s="12" t="inlineStr">
         <is>
           <t>final_model_path</t>
         </is>
       </c>
-      <c r="BC1" s="12" t="inlineStr">
+      <c r="BF1" s="12" t="inlineStr">
         <is>
           <t>final_model_type</t>
         </is>
@@ -10175,17 +10500,20 @@
       <c r="AX2" s="13" t="inlineStr"/>
       <c r="AY2" s="13" t="inlineStr"/>
       <c r="AZ2" s="13" t="inlineStr"/>
-      <c r="BA2" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BB2" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BC2" s="13" t="inlineStr">
+      <c r="BA2" s="13" t="inlineStr"/>
+      <c r="BB2" s="13" t="inlineStr"/>
+      <c r="BC2" s="13" t="inlineStr"/>
+      <c r="BD2" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE2" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BF2" s="13" t="inlineStr">
         <is>
           <t>single</t>
         </is>
@@ -10424,17 +10752,20 @@
         </is>
       </c>
       <c r="AZ3" s="17" t="inlineStr"/>
-      <c r="BA3" s="16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BB3" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BC3" s="17" t="inlineStr">
+      <c r="BA3" s="17" t="inlineStr"/>
+      <c r="BB3" s="17" t="inlineStr"/>
+      <c r="BC3" s="17" t="inlineStr"/>
+      <c r="BD3" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE3" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BF3" s="17" t="inlineStr">
         <is>
           <t>single</t>
         </is>
@@ -10673,17 +11004,20 @@
         </is>
       </c>
       <c r="AZ4" s="13" t="inlineStr"/>
-      <c r="BA4" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BB4" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BC4" s="13" t="inlineStr">
+      <c r="BA4" s="13" t="inlineStr"/>
+      <c r="BB4" s="13" t="inlineStr"/>
+      <c r="BC4" s="13" t="inlineStr"/>
+      <c r="BD4" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE4" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BF4" s="13" t="inlineStr">
         <is>
           <t>single</t>
         </is>
@@ -10914,17 +11248,20 @@
       <c r="AX5" s="17" t="inlineStr"/>
       <c r="AY5" s="17" t="inlineStr"/>
       <c r="AZ5" s="17" t="inlineStr"/>
-      <c r="BA5" s="16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BB5" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BC5" s="17" t="inlineStr">
+      <c r="BA5" s="17" t="inlineStr"/>
+      <c r="BB5" s="17" t="inlineStr"/>
+      <c r="BC5" s="17" t="inlineStr"/>
+      <c r="BD5" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE5" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BF5" s="17" t="inlineStr">
         <is>
           <t>single</t>
         </is>
@@ -11171,17 +11508,20 @@
       <c r="AX6" s="13" t="inlineStr"/>
       <c r="AY6" s="13" t="inlineStr"/>
       <c r="AZ6" s="13" t="inlineStr"/>
-      <c r="BA6" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BB6" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BC6" s="13" t="inlineStr">
+      <c r="BA6" s="13" t="inlineStr"/>
+      <c r="BB6" s="13" t="inlineStr"/>
+      <c r="BC6" s="13" t="inlineStr"/>
+      <c r="BD6" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE6" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BF6" s="13" t="inlineStr">
         <is>
           <t>best_complete</t>
         </is>
@@ -11408,13 +11748,16 @@
           <t>open</t>
         </is>
       </c>
-      <c r="BA7" s="19" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="BA7" s="17" t="inlineStr"/>
       <c r="BB7" s="17" t="inlineStr"/>
       <c r="BC7" s="17" t="inlineStr"/>
+      <c r="BD7" s="19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BE7" s="17" t="inlineStr"/>
+      <c r="BF7" s="17" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="21" t="inlineStr">
@@ -11637,13 +11980,16 @@
           <t>open</t>
         </is>
       </c>
-      <c r="BA8" s="21" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="BA8" s="13" t="inlineStr"/>
       <c r="BB8" s="13" t="inlineStr"/>
       <c r="BC8" s="13" t="inlineStr"/>
+      <c r="BD8" s="21" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BE8" s="13" t="inlineStr"/>
+      <c r="BF8" s="13" t="inlineStr"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="16" t="inlineStr">
@@ -11890,17 +12236,20 @@
       <c r="AX9" s="17" t="inlineStr"/>
       <c r="AY9" s="17" t="inlineStr"/>
       <c r="AZ9" s="17" t="inlineStr"/>
-      <c r="BA9" s="16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BB9" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BC9" s="17" t="inlineStr">
+      <c r="BA9" s="17" t="inlineStr"/>
+      <c r="BB9" s="17" t="inlineStr"/>
+      <c r="BC9" s="17" t="inlineStr"/>
+      <c r="BD9" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE9" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BF9" s="17" t="inlineStr">
         <is>
           <t>gaps,large_gap_complete</t>
         </is>
@@ -12115,13 +12464,16 @@
       <c r="AX10" s="13" t="inlineStr"/>
       <c r="AY10" s="13" t="inlineStr"/>
       <c r="AZ10" s="13" t="inlineStr"/>
-      <c r="BA10" s="21" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="BA10" s="13" t="inlineStr"/>
       <c r="BB10" s="13" t="inlineStr"/>
       <c r="BC10" s="13" t="inlineStr"/>
+      <c r="BD10" s="21" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BE10" s="13" t="inlineStr"/>
+      <c r="BF10" s="13" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="16" t="inlineStr">
@@ -12364,17 +12716,20 @@
       <c r="AX11" s="17" t="inlineStr"/>
       <c r="AY11" s="17" t="inlineStr"/>
       <c r="AZ11" s="17" t="inlineStr"/>
-      <c r="BA11" s="16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BB11" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BC11" s="17" t="inlineStr">
+      <c r="BA11" s="17" t="inlineStr"/>
+      <c r="BB11" s="17" t="inlineStr"/>
+      <c r="BC11" s="17" t="inlineStr"/>
+      <c r="BD11" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE11" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BF11" s="17" t="inlineStr">
         <is>
           <t>best_complete</t>
         </is>
@@ -12625,17 +12980,32 @@
       <c r="AX12" s="13" t="inlineStr"/>
       <c r="AY12" s="13" t="inlineStr"/>
       <c r="AZ12" s="13" t="inlineStr"/>
-      <c r="BA12" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BB12" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BC12" s="13" t="inlineStr">
+      <c r="BA12" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="BB12" s="13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BC12" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BD12" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE12" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BF12" s="13" t="inlineStr">
         <is>
           <t>gaps,best_complete</t>
         </is>
@@ -12862,13 +13232,16 @@
           <t>open</t>
         </is>
       </c>
-      <c r="BA13" s="19" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="BA13" s="17" t="inlineStr"/>
       <c r="BB13" s="17" t="inlineStr"/>
       <c r="BC13" s="17" t="inlineStr"/>
+      <c r="BD13" s="19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BE13" s="17" t="inlineStr"/>
+      <c r="BF13" s="17" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -13111,17 +13484,20 @@
       <c r="AX14" s="13" t="inlineStr"/>
       <c r="AY14" s="13" t="inlineStr"/>
       <c r="AZ14" s="13" t="inlineStr"/>
-      <c r="BA14" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BB14" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BC14" s="13" t="inlineStr">
+      <c r="BA14" s="13" t="inlineStr"/>
+      <c r="BB14" s="13" t="inlineStr"/>
+      <c r="BC14" s="13" t="inlineStr"/>
+      <c r="BD14" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE14" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BF14" s="13" t="inlineStr">
         <is>
           <t>best_complete</t>
         </is>
@@ -13348,13 +13724,16 @@
           <t>open</t>
         </is>
       </c>
-      <c r="BA15" s="19" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="BA15" s="17" t="inlineStr"/>
       <c r="BB15" s="17" t="inlineStr"/>
       <c r="BC15" s="17" t="inlineStr"/>
+      <c r="BD15" s="19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BE15" s="17" t="inlineStr"/>
+      <c r="BF15" s="17" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -13593,17 +13972,20 @@
         </is>
       </c>
       <c r="AZ16" s="13" t="inlineStr"/>
-      <c r="BA16" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BB16" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BC16" s="13" t="inlineStr">
+      <c r="BA16" s="13" t="inlineStr"/>
+      <c r="BB16" s="13" t="inlineStr"/>
+      <c r="BC16" s="13" t="inlineStr"/>
+      <c r="BD16" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE16" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BF16" s="13" t="inlineStr">
         <is>
           <t>gaps</t>
         </is>
@@ -13834,17 +14216,20 @@
       <c r="AX17" s="17" t="inlineStr"/>
       <c r="AY17" s="17" t="inlineStr"/>
       <c r="AZ17" s="17" t="inlineStr"/>
-      <c r="BA17" s="16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BB17" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BC17" s="17" t="inlineStr">
+      <c r="BA17" s="17" t="inlineStr"/>
+      <c r="BB17" s="17" t="inlineStr"/>
+      <c r="BC17" s="17" t="inlineStr"/>
+      <c r="BD17" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE17" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BF17" s="17" t="inlineStr">
         <is>
           <t>single</t>
         </is>
@@ -14059,13 +14444,16 @@
       <c r="AX18" s="13" t="inlineStr"/>
       <c r="AY18" s="13" t="inlineStr"/>
       <c r="AZ18" s="13" t="inlineStr"/>
-      <c r="BA18" s="21" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="BA18" s="13" t="inlineStr"/>
       <c r="BB18" s="13" t="inlineStr"/>
       <c r="BC18" s="13" t="inlineStr"/>
+      <c r="BD18" s="21" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BE18" s="13" t="inlineStr"/>
+      <c r="BF18" s="13" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
@@ -14312,17 +14700,32 @@
       <c r="AX19" s="17" t="inlineStr"/>
       <c r="AY19" s="17" t="inlineStr"/>
       <c r="AZ19" s="17" t="inlineStr"/>
-      <c r="BA19" s="16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BB19" s="30" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BC19" s="17" t="inlineStr">
+      <c r="BA19" s="15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="BB19" s="17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BC19" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BD19" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE19" s="30" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BF19" s="17" t="inlineStr">
         <is>
           <t>gaps,best_complete</t>
         </is>
@@ -14553,17 +14956,20 @@
       <c r="AX20" s="13" t="inlineStr"/>
       <c r="AY20" s="13" t="inlineStr"/>
       <c r="AZ20" s="13" t="inlineStr"/>
-      <c r="BA20" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="BB20" s="29" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="BC20" s="13" t="inlineStr">
+      <c r="BA20" s="13" t="inlineStr"/>
+      <c r="BB20" s="13" t="inlineStr"/>
+      <c r="BC20" s="13" t="inlineStr"/>
+      <c r="BD20" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE20" s="29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="BF20" s="13" t="inlineStr">
         <is>
           <t>single</t>
         </is>
@@ -14786,16 +15192,19 @@
         </is>
       </c>
       <c r="AZ21" s="17" t="inlineStr"/>
-      <c r="BA21" s="19" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="BA21" s="17" t="inlineStr"/>
       <c r="BB21" s="17" t="inlineStr"/>
       <c r="BC21" s="17" t="inlineStr"/>
+      <c r="BD21" s="19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BE21" s="17" t="inlineStr"/>
+      <c r="BF21" s="17" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BC21"/>
+  <autoFilter ref="A1:BF21"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
@@ -14808,7 +15217,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE2" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV2" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW2" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB2" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BE2" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId15"/>
@@ -14821,7 +15230,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV3" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW3" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY3" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB3" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BE3" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId28"/>
@@ -14834,7 +15243,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV4" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW4" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY4" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB4" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BE4" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId41"/>
@@ -14846,7 +15255,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE5" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV5" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW5" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB5" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BE5" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId53"/>
@@ -14861,7 +15270,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL6" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV6" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW6" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB6" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BE6" r:id="rId65"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId68"/>
@@ -14899,7 +15308,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL9" r:id="rId100"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV9" r:id="rId101"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW9" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB9" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BE9" r:id="rId103"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId104"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId105"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId106"/>
@@ -14923,7 +15332,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL11" r:id="rId124"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV11" r:id="rId125"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW11" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB11" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BE11" r:id="rId127"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId128"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId129"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId130"/>
@@ -14939,117 +15348,119 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK12" r:id="rId140"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV12" r:id="rId141"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW12" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB12" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y13" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z13" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV13" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW13" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY13" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ13" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U14" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y14" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z14" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD14" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE14" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL14" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV14" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW14" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB14" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y15" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z15" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV15" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW15" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY15" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ15" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y16" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z16" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD16" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE16" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ16" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV16" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW16" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY16" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB16" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y17" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z17" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD17" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE17" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV17" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW17" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB17" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y18" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z18" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV18" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW18" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U19" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y19" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z19" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD19" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE19" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ19" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL19" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV19" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW19" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB19" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y20" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z20" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD20" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE20" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV20" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW20" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BB20" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y21" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z21" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV21" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW21" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY21" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BC12" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BE12" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y13" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z13" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV13" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW13" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY13" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ13" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U14" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y14" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z14" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD14" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE14" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL14" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV14" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW14" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BE14" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y15" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z15" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV15" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW15" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY15" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ15" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y16" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z16" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD16" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE16" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ16" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV16" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW16" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY16" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BE16" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y17" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z17" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD17" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE17" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV17" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW17" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BE17" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y18" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z18" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV18" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW18" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U19" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y19" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z19" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD19" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE19" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ19" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL19" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV19" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW19" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BC19" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BE19" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y20" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z20" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD20" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE20" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV20" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW20" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="BE20" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y21" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z21" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AV21" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW21" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY21" r:id="rId255"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>